<commit_message>
Update company radar data
</commit_message>
<xml_diff>
--- a/company_radar_output.xlsx
+++ b/company_radar_output.xlsx
@@ -1024,16 +1024,16 @@
         <v>453.1150103759766</v>
       </c>
       <c r="AG3" t="n">
-        <v>429.6539505004883</v>
+        <v>429.6539512634278</v>
       </c>
       <c r="AH3" t="n">
         <v>0.09382826331786864</v>
       </c>
       <c r="AI3" t="n">
-        <v>0.1535562615110861</v>
+        <v>0.1535562594627082</v>
       </c>
       <c r="AJ3" t="n">
-        <v>0.05460454826066274</v>
+        <v>0.05460454638799406</v>
       </c>
       <c r="AK3" t="n">
         <v>537.6464233398438</v>
@@ -1072,13 +1072,13 @@
         <v>-0.002599009870587476</v>
       </c>
       <c r="AW3" t="n">
-        <v>0.7149102799980402</v>
+        <v>0.7149095556703464</v>
       </c>
       <c r="AX3" t="n">
         <v>0.05462505519623884</v>
       </c>
       <c r="AY3" t="n">
-        <v>8397.480698943207</v>
+        <v>8397.481229099616</v>
       </c>
       <c r="AZ3" t="inlineStr"/>
       <c r="BA3" t="n">
@@ -1268,13 +1268,13 @@
         <v>1.957717803516736</v>
       </c>
       <c r="AW4" t="n">
-        <v>4.206413767596303</v>
+        <v>4.206412941685683</v>
       </c>
       <c r="AX4" t="n">
         <v>2.321982329146867</v>
       </c>
       <c r="AY4" t="n">
-        <v>4.251978127284558</v>
+        <v>4.251977707069563</v>
       </c>
       <c r="AZ4" t="inlineStr"/>
       <c r="BA4" t="n">
@@ -1416,16 +1416,16 @@
         <v>600.902197265625</v>
       </c>
       <c r="AG5" t="n">
-        <v>622.5782839965821</v>
+        <v>622.5782849121093</v>
       </c>
       <c r="AH5" t="n">
         <v>0.07842845681993316</v>
       </c>
       <c r="AI5" t="n">
-        <v>0.04088119671779733</v>
+        <v>0.04088119518713818</v>
       </c>
       <c r="AJ5" t="n">
-        <v>-0.03481664440945398</v>
+        <v>-0.03481664582879629</v>
       </c>
       <c r="AK5" t="n">
         <v>777.7011108398438</v>
@@ -1461,16 +1461,16 @@
         <v>0.05780582477842255</v>
       </c>
       <c r="AV5" t="n">
-        <v>-0.1341670638786125</v>
+        <v>-0.1341671344864807</v>
       </c>
       <c r="AW5" t="n">
-        <v>0.7374177085686509</v>
+        <v>0.737417566413243</v>
       </c>
       <c r="AX5" t="n">
         <v>-0.001881861088982584</v>
       </c>
       <c r="AY5" t="n">
-        <v>16.09968370898972</v>
+        <v>16.09967854527519</v>
       </c>
       <c r="AZ5" t="inlineStr"/>
       <c r="BA5" t="n">
@@ -1612,16 +1612,16 @@
         <v>346.9777496337891</v>
       </c>
       <c r="AG6" t="n">
-        <v>336.3809658813477</v>
+        <v>336.3809657287597</v>
       </c>
       <c r="AH6" t="n">
         <v>-0.02443312184350943</v>
       </c>
       <c r="AI6" t="n">
-        <v>0.006299506611797456</v>
+        <v>0.006299507068271204</v>
       </c>
       <c r="AJ6" t="n">
-        <v>0.03150232869055736</v>
+        <v>0.03150232915846374</v>
       </c>
       <c r="AK6" t="n">
         <v>402.1211853027344</v>
@@ -1657,10 +1657,10 @@
         <v>0.1212118179624675</v>
       </c>
       <c r="AV6" t="n">
-        <v>0.4119079606978782</v>
+        <v>0.4119080505594885</v>
       </c>
       <c r="AW6" t="n">
-        <v>1.377363626445911</v>
+        <v>1.377363881218482</v>
       </c>
       <c r="AX6" t="n">
         <v>0.07618107138345542</v>
@@ -1773,7 +1773,7 @@
         </is>
       </c>
       <c r="X7" t="n">
-        <v>61045092352</v>
+        <v>57012838400</v>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
@@ -1784,7 +1784,7 @@
         <v>1</v>
       </c>
       <c r="AA7" t="n">
-        <v>61045092352</v>
+        <v>57012838400</v>
       </c>
       <c r="AB7" t="inlineStr">
         <is>
@@ -2384,16 +2384,16 @@
         <v>140.6299467468262</v>
       </c>
       <c r="AG10" t="n">
-        <v>166.8175089645386</v>
+        <v>166.8175086593628</v>
       </c>
       <c r="AH10" t="n">
         <v>0.06862017838806089</v>
       </c>
       <c r="AI10" t="n">
-        <v>-0.09913533829807508</v>
+        <v>-0.09913533665003416</v>
       </c>
       <c r="AJ10" t="n">
-        <v>-0.1569832949806201</v>
+        <v>-0.1569832934384063</v>
       </c>
       <c r="AK10" t="n">
         <v>324.4519958496094</v>
@@ -2429,16 +2429,16 @@
         <v>-0.02437296863035288</v>
       </c>
       <c r="AV10" t="n">
-        <v>-0.5062923382987412</v>
+        <v>-0.5062922888006263</v>
       </c>
       <c r="AW10" t="n">
-        <v>0.7862063968632773</v>
+        <v>0.7862065588398521</v>
       </c>
       <c r="AX10" t="n">
-        <v>-0.2247226929797956</v>
+        <v>-0.2247226319512438</v>
       </c>
       <c r="AY10" t="n">
-        <v>2990.385372388566</v>
+        <v>2990.384485102764</v>
       </c>
       <c r="AZ10" t="inlineStr"/>
       <c r="BA10" t="n">
@@ -2624,13 +2624,13 @@
         <v>-0.275870939666826</v>
       </c>
       <c r="AW11" t="n">
-        <v>0.08255307053061633</v>
+        <v>0.0825529870474393</v>
       </c>
       <c r="AX11" t="n">
         <v>-0.3043479187343738</v>
       </c>
       <c r="AY11" t="n">
-        <v>608.1361819570965</v>
+        <v>608.1362852069659</v>
       </c>
       <c r="AZ11" t="inlineStr"/>
       <c r="BA11" t="n">
@@ -2816,13 +2816,13 @@
         <v>-0.2903769299056658</v>
       </c>
       <c r="AW12" t="n">
-        <v>-0.3179885595200022</v>
+        <v>-0.3179884945843425</v>
       </c>
       <c r="AX12" t="n">
         <v>-0.291743876346652</v>
       </c>
       <c r="AY12" t="n">
-        <v>0.2370492813136365</v>
+        <v>0.2370493881315128</v>
       </c>
       <c r="AZ12" t="inlineStr"/>
       <c r="BA12" t="n">
@@ -3121,7 +3121,7 @@
         </is>
       </c>
       <c r="X14" t="n">
-        <v>14821988352</v>
+        <v>14759337984</v>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
@@ -3132,7 +3132,7 @@
         <v>1</v>
       </c>
       <c r="AA14" t="n">
-        <v>14821988352</v>
+        <v>14759337984</v>
       </c>
       <c r="AB14" t="inlineStr">
         <is>
@@ -3901,7 +3901,7 @@
         </is>
       </c>
       <c r="X18" t="n">
-        <v>29133248512</v>
+        <v>29178312704</v>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
@@ -3912,7 +3912,7 @@
         <v>1</v>
       </c>
       <c r="AA18" t="n">
-        <v>29133248512</v>
+        <v>29178312704</v>
       </c>
       <c r="AB18" t="inlineStr">
         <is>
@@ -4755,16 +4755,16 @@
         <v>0.1277732642630893</v>
       </c>
       <c r="AV22" t="n">
-        <v>0.01393743323475483</v>
+        <v>0.01393734656336121</v>
       </c>
       <c r="AW22" t="n">
-        <v>6.989548382805551</v>
+        <v>6.989549055484776</v>
       </c>
       <c r="AX22" t="n">
         <v>0.0451742685812544</v>
       </c>
       <c r="AY22" t="n">
-        <v>317.767752326703</v>
+        <v>317.7679865664864</v>
       </c>
       <c r="AZ22" t="inlineStr"/>
       <c r="BA22" t="n">
@@ -4906,16 +4906,16 @@
         <v>237.1030813598633</v>
       </c>
       <c r="AG23" t="n">
-        <v>258.0273531341552</v>
+        <v>258.0273535919189</v>
       </c>
       <c r="AH23" t="n">
         <v>0.02609376432725208</v>
       </c>
       <c r="AI23" t="n">
-        <v>-0.05711549441953967</v>
+        <v>-0.05711549609230138</v>
       </c>
       <c r="AJ23" t="n">
-        <v>-0.08109323108629063</v>
+        <v>-0.08109323271651381</v>
       </c>
       <c r="AK23" t="n">
         <v>326.8851013183594</v>
@@ -4951,16 +4951,16 @@
         <v>0.002268520599327362</v>
       </c>
       <c r="AV23" t="n">
-        <v>-0.02877417944781357</v>
+        <v>-0.02877412028670689</v>
       </c>
       <c r="AW23" t="n">
-        <v>1.207604887086692</v>
+        <v>1.20760503991667</v>
       </c>
       <c r="AX23" t="n">
-        <v>-0.1483840812308197</v>
+        <v>-0.1483841722039867</v>
       </c>
       <c r="AY23" t="n">
-        <v>168.6051232295094</v>
+        <v>168.6051514194302</v>
       </c>
       <c r="AZ23" t="inlineStr"/>
       <c r="BA23" t="n">
@@ -5093,7 +5093,7 @@
         <v>29567</v>
       </c>
       <c r="AD24" t="n">
-        <v>45.7</v>
+        <v>45.8</v>
       </c>
       <c r="AE24" t="n">
         <v>332.2699890136719</v>
@@ -5102,16 +5102,16 @@
         <v>317.8303741455078</v>
       </c>
       <c r="AG24" t="n">
-        <v>284.5368991851807</v>
+        <v>284.5368969726562</v>
       </c>
       <c r="AH24" t="n">
         <v>0.0454318279270356</v>
       </c>
       <c r="AI24" t="n">
-        <v>0.1677571167928762</v>
+        <v>0.1677571258732142</v>
       </c>
       <c r="AJ24" t="n">
-        <v>0.1170093406362007</v>
+        <v>0.1170093493219302</v>
       </c>
       <c r="AK24" t="n">
         <v>339.7869262695312</v>
@@ -5150,13 +5150,13 @@
         <v>0.4497995740678464</v>
       </c>
       <c r="AW24" t="n">
-        <v>1.207777594829726</v>
+        <v>1.207776699466175</v>
       </c>
       <c r="AX24" t="n">
-        <v>0.2293803880831269</v>
+        <v>0.2293805268965801</v>
       </c>
       <c r="AY24" t="n">
-        <v>3385.280334952015</v>
+        <v>3385.281363453541</v>
       </c>
       <c r="AZ24" t="inlineStr"/>
       <c r="BA24" t="n">
@@ -5490,16 +5490,16 @@
         <v>212.3561532592773</v>
       </c>
       <c r="AG26" t="n">
-        <v>197.1051929473877</v>
+        <v>197.1051928710937</v>
       </c>
       <c r="AH26" t="n">
         <v>0.02794286831712633</v>
       </c>
       <c r="AI26" t="n">
-        <v>0.1074796661719606</v>
+        <v>0.1074796666006352</v>
       </c>
       <c r="AJ26" t="n">
-        <v>0.07737472607309992</v>
+        <v>0.07737472649012189</v>
       </c>
       <c r="AK26" t="n">
         <v>235.202392578125</v>
@@ -5532,19 +5532,19 @@
         <v>0.06503360332428509</v>
       </c>
       <c r="AU26" t="n">
-        <v>0.2138082500949225</v>
+        <v>0.2138083530828809</v>
       </c>
       <c r="AV26" t="n">
-        <v>0.2350453814344682</v>
+        <v>0.2350452748111889</v>
       </c>
       <c r="AW26" t="n">
-        <v>8.598190240151791</v>
+        <v>8.598189435190632</v>
       </c>
       <c r="AX26" t="n">
         <v>0.1585955986034835</v>
       </c>
       <c r="AY26" t="n">
-        <v>5817.413780112818</v>
+        <v>5817.41435785695</v>
       </c>
       <c r="AZ26" t="inlineStr"/>
       <c r="BA26" t="n">
@@ -5855,10 +5855,10 @@
         </is>
       </c>
       <c r="Z28" t="n">
-        <v>0.1490868479013443</v>
+        <v>0.1490846127271652</v>
       </c>
       <c r="AA28" t="n">
-        <v>97504019388.94238</v>
+        <v>97502557566.72559</v>
       </c>
       <c r="AB28" t="inlineStr">
         <is>
@@ -6316,13 +6316,13 @@
         <v>3.182852494449236</v>
       </c>
       <c r="AW30" t="n">
-        <v>1.088626622413908</v>
+        <v>1.0886264607558</v>
       </c>
       <c r="AX30" t="n">
         <v>1.614017258743895</v>
       </c>
       <c r="AY30" t="n">
-        <v>566.1632843449839</v>
+        <v>566.1632377807866</v>
       </c>
       <c r="AZ30" t="inlineStr"/>
       <c r="BA30" t="n">
@@ -6455,7 +6455,7 @@
         <v>33585</v>
       </c>
       <c r="AD31" t="n">
-        <v>34.7</v>
+        <v>34.8</v>
       </c>
       <c r="AE31" t="n">
         <v>181.9700012207031</v>
@@ -6464,28 +6464,28 @@
         <v>167.8024603271484</v>
       </c>
       <c r="AG31" t="n">
-        <v>166.4593501281738</v>
+        <v>166.4593502426147</v>
       </c>
       <c r="AH31" t="n">
         <v>0.0844298758548212</v>
       </c>
       <c r="AI31" t="n">
-        <v>0.09317981285272392</v>
+        <v>0.09317981210116222</v>
       </c>
       <c r="AJ31" t="n">
-        <v>0.008068697840886596</v>
+        <v>0.008068697147838755</v>
       </c>
       <c r="AK31" t="n">
-        <v>248.7424926757812</v>
+        <v>248.7425079345703</v>
       </c>
       <c r="AL31" t="n">
-        <v>122.9443130493164</v>
+        <v>122.9443054199219</v>
       </c>
       <c r="AM31" t="n">
-        <v>-0.2684402280317721</v>
+        <v>-0.2684402729083649</v>
       </c>
       <c r="AN31" t="n">
-        <v>0.4801010043279501</v>
+        <v>0.4801010961766492</v>
       </c>
       <c r="AO31" t="n">
         <v>80.41228104081972</v>
@@ -6509,16 +6509,16 @@
         <v>0.4145441441817588</v>
       </c>
       <c r="AV31" t="n">
-        <v>0.1501423840060041</v>
+        <v>0.1501424949294952</v>
       </c>
       <c r="AW31" t="n">
-        <v>0.4026838698810877</v>
+        <v>0.402683539914648</v>
       </c>
       <c r="AX31" t="n">
         <v>0.06841928392637908</v>
       </c>
       <c r="AY31" t="n">
-        <v>541.2931196477541</v>
+        <v>541.2933123020266</v>
       </c>
       <c r="AZ31" t="inlineStr"/>
       <c r="BA31" t="n">
@@ -6704,7 +6704,7 @@
         <v>6.804807488360287</v>
       </c>
       <c r="AW32" t="n">
-        <v>4.242268784622484</v>
+        <v>4.242268274485537</v>
       </c>
       <c r="AX32" t="n">
         <v>4.278251218089809</v>
@@ -6900,7 +6900,7 @@
         <v>2.588393791907249</v>
       </c>
       <c r="AW33" t="n">
-        <v>4.441159917053373</v>
+        <v>4.44116027472621</v>
       </c>
       <c r="AX33" t="n">
         <v>1.364593793492743</v>
@@ -7098,7 +7098,7 @@
         <v>1.737572926819951</v>
       </c>
       <c r="AY34" t="n">
-        <v>27.26115241316053</v>
+        <v>27.26115988990115</v>
       </c>
       <c r="AZ34" t="inlineStr"/>
       <c r="BA34" t="n">
@@ -7284,13 +7284,13 @@
         <v>6.278814266453553</v>
       </c>
       <c r="AW35" t="n">
-        <v>6.661409185290411</v>
+        <v>6.66141010202343</v>
       </c>
       <c r="AX35" t="n">
         <v>3.470322288087283</v>
       </c>
       <c r="AY35" t="n">
-        <v>133.2129188640086</v>
+        <v>133.2129100724851</v>
       </c>
       <c r="AZ35" t="inlineStr"/>
       <c r="BA35" t="n">
@@ -7405,10 +7405,10 @@
         </is>
       </c>
       <c r="Z36" t="n">
-        <v>1.160227417945862</v>
+        <v>1.160092830657959</v>
       </c>
       <c r="AA36" t="n">
-        <v>7500452575.149536</v>
+        <v>7499582516.784668</v>
       </c>
       <c r="AB36" t="inlineStr">
         <is>
@@ -7476,13 +7476,13 @@
         <v>7.822905011209466</v>
       </c>
       <c r="AW36" t="n">
-        <v>4.293791511379664</v>
+        <v>4.2937918326055</v>
       </c>
       <c r="AX36" t="n">
         <v>4.073170663628245</v>
       </c>
       <c r="AY36" t="n">
-        <v>13.50121847008162</v>
+        <v>13.50121967527242</v>
       </c>
       <c r="AZ36" t="inlineStr"/>
       <c r="BA36" t="n">
@@ -7785,7 +7785,7 @@
         </is>
       </c>
       <c r="X38" t="n">
-        <v>12852446208</v>
+        <v>12822445056</v>
       </c>
       <c r="Y38" t="inlineStr">
         <is>
@@ -7796,7 +7796,7 @@
         <v>1</v>
       </c>
       <c r="AA38" t="n">
-        <v>12852446208</v>
+        <v>12822445056</v>
       </c>
       <c r="AB38" t="inlineStr">
         <is>
@@ -7816,16 +7816,16 @@
         <v>56.28073356628418</v>
       </c>
       <c r="AG38" t="n">
-        <v>56.32725648880005</v>
+        <v>56.32725671768188</v>
       </c>
       <c r="AH38" t="n">
         <v>-0.08085775958638242</v>
       </c>
       <c r="AI38" t="n">
-        <v>-0.08161691573737173</v>
+        <v>-0.08161691946915661</v>
       </c>
       <c r="AJ38" t="n">
-        <v>-0.0008259397921345224</v>
+        <v>-0.000825943852207911</v>
       </c>
       <c r="AK38" t="n">
         <v>93.37815856933594</v>
@@ -7867,7 +7867,7 @@
         <v>0.9479422416482752</v>
       </c>
       <c r="AX38" t="n">
-        <v>0.2111586717106346</v>
+        <v>0.2111587798838475</v>
       </c>
       <c r="AY38" t="n">
         <v>3.190138934003741</v>
@@ -8056,13 +8056,13 @@
         <v>0.2107603892268155</v>
       </c>
       <c r="AW39" t="n">
-        <v>1.044324296820654</v>
+        <v>1.044324465136008</v>
       </c>
       <c r="AX39" t="n">
         <v>0.1253661186097392</v>
       </c>
       <c r="AY39" t="n">
-        <v>3.632144345582888</v>
+        <v>3.632143049360775</v>
       </c>
       <c r="AZ39" t="inlineStr"/>
       <c r="BA39" t="n">
@@ -8169,7 +8169,7 @@
         </is>
       </c>
       <c r="X40" t="n">
-        <v>14236608626688</v>
+        <v>14267368603648</v>
       </c>
       <c r="Y40" t="inlineStr">
         <is>
@@ -8180,7 +8180,7 @@
         <v>0.00651236716657877</v>
       </c>
       <c r="AA40" t="n">
-        <v>92714022583.875</v>
+        <v>92914342847.87402</v>
       </c>
       <c r="AB40" t="inlineStr">
         <is>
@@ -8396,16 +8396,16 @@
         <v>187.0133999633789</v>
       </c>
       <c r="AG41" t="n">
-        <v>178.1654887390137</v>
+        <v>178.1654884338379</v>
       </c>
       <c r="AH41" t="n">
         <v>0.008376949822753721</v>
       </c>
       <c r="AI41" t="n">
-        <v>0.05845415498675366</v>
+        <v>0.05845415679975674</v>
       </c>
       <c r="AJ41" t="n">
-        <v>0.04966119581849049</v>
+        <v>0.04966119761643228</v>
       </c>
       <c r="AK41" t="n">
         <v>202.5594635009766</v>
@@ -8441,16 +8441,16 @@
         <v>0.05694186929571288</v>
       </c>
       <c r="AV41" t="n">
-        <v>0.1108041317727211</v>
+        <v>0.1108042316115425</v>
       </c>
       <c r="AW41" t="n">
-        <v>0.3345997084972185</v>
+        <v>0.3346002849804299</v>
       </c>
       <c r="AX41" t="n">
         <v>0.2328575223559801</v>
       </c>
       <c r="AY41" t="n">
-        <v>35.99377267965599</v>
+        <v>35.99376921921329</v>
       </c>
       <c r="AZ41" t="inlineStr"/>
       <c r="BA41" t="n">
@@ -8637,10 +8637,10 @@
         <v>0.08035399408722066</v>
       </c>
       <c r="AV42" t="n">
-        <v>0.3290945945840307</v>
+        <v>0.3290944906849667</v>
       </c>
       <c r="AW42" t="n">
-        <v>0.2985354628332308</v>
+        <v>0.2985351653046637</v>
       </c>
       <c r="AX42" t="n">
         <v>0.3787888605369425</v>
@@ -8788,28 +8788,28 @@
         <v>121.4274002075195</v>
       </c>
       <c r="AG43" t="n">
-        <v>109.3037474060059</v>
+        <v>109.3037472915649</v>
       </c>
       <c r="AH43" t="n">
         <v>-0.05144967191644501</v>
       </c>
       <c r="AI43" t="n">
-        <v>0.05376076336470637</v>
+        <v>0.05376076446799294</v>
       </c>
       <c r="AJ43" t="n">
-        <v>0.1109170828012025</v>
+        <v>0.1109170839643314</v>
       </c>
       <c r="AK43" t="n">
         <v>133.0599975585938</v>
       </c>
       <c r="AL43" t="n">
-        <v>77.69111633300781</v>
+        <v>77.69110870361328</v>
       </c>
       <c r="AM43" t="n">
         <v>-0.1343754515367731</v>
       </c>
       <c r="AN43" t="n">
-        <v>0.4825375891302577</v>
+        <v>0.4825377347178847</v>
       </c>
       <c r="AO43" t="n">
         <v>36.33094490431546</v>
@@ -8839,10 +8839,10 @@
         <v>1.834340358383641</v>
       </c>
       <c r="AX43" t="n">
-        <v>0.4045281691811533</v>
+        <v>0.4045280385117627</v>
       </c>
       <c r="AY43" t="n">
-        <v>98.96806774073896</v>
+        <v>98.96802636788964</v>
       </c>
       <c r="AZ43" t="inlineStr"/>
       <c r="BA43" t="n">
@@ -8980,28 +8980,28 @@
         <v>2.18869544506073</v>
       </c>
       <c r="AG44" t="n">
-        <v>2.173684566020965</v>
+        <v>2.173684567213058</v>
       </c>
       <c r="AH44" t="n">
         <v>-0.02224856832705846</v>
       </c>
       <c r="AI44" t="n">
-        <v>-0.01549648078812627</v>
+        <v>-0.01549648132804815</v>
       </c>
       <c r="AJ44" t="n">
-        <v>0.006905730147977573</v>
+        <v>0.00690572959576996</v>
       </c>
       <c r="AK44" t="n">
         <v>2.30321192741394</v>
       </c>
       <c r="AL44" t="n">
-        <v>2.061682462692261</v>
+        <v>2.061682224273682</v>
       </c>
       <c r="AM44" t="n">
         <v>-0.07086270289205254</v>
       </c>
       <c r="AN44" t="n">
-        <v>0.03798724761408812</v>
+        <v>0.03798736764977639</v>
       </c>
       <c r="AO44" t="n">
         <v>25.67112826337086</v>
@@ -9028,13 +9028,13 @@
         <v>-0.03678298057557294</v>
       </c>
       <c r="AW44" t="n">
-        <v>0.06435019376538054</v>
+        <v>0.06435006755492445</v>
       </c>
       <c r="AX44" t="n">
         <v>0.01481794284745197</v>
       </c>
       <c r="AY44" t="n">
-        <v>2.977313856374117</v>
+        <v>2.977314737577442</v>
       </c>
       <c r="AZ44" t="inlineStr"/>
       <c r="BA44" t="n">
@@ -9163,7 +9163,7 @@
         <v>40525</v>
       </c>
       <c r="AD45" t="n">
-        <v>15.7</v>
+        <v>15.8</v>
       </c>
       <c r="AE45" t="n">
         <v>12.0600004196167</v>
@@ -9709,7 +9709,7 @@
         </is>
       </c>
       <c r="X48" t="n">
-        <v>1993217015808</v>
+        <v>1992068956160</v>
       </c>
       <c r="Y48" t="inlineStr">
         <is>
@@ -9720,7 +9720,7 @@
         <v>1</v>
       </c>
       <c r="AA48" t="n">
-        <v>1993217015808</v>
+        <v>1992068956160</v>
       </c>
       <c r="AB48" t="inlineStr">
         <is>
@@ -9891,7 +9891,7 @@
         </is>
       </c>
       <c r="X49" t="n">
-        <v>10551757824</v>
+        <v>10547602432</v>
       </c>
       <c r="Y49" t="inlineStr">
         <is>
@@ -9902,7 +9902,7 @@
         <v>1</v>
       </c>
       <c r="AA49" t="n">
-        <v>10551757824</v>
+        <v>10547602432</v>
       </c>
       <c r="AB49" t="inlineStr">
         <is>
@@ -9937,13 +9937,13 @@
         <v>16.86722755432129</v>
       </c>
       <c r="AL49" t="n">
-        <v>11.91677379608154</v>
+        <v>11.91677284240723</v>
       </c>
       <c r="AM49" t="n">
         <v>-0.1231516908026825</v>
       </c>
       <c r="AN49" t="n">
-        <v>0.24110772050706</v>
+        <v>0.2411078198303056</v>
       </c>
       <c r="AO49" t="n">
         <v>53.8460127717481</v>
@@ -9970,13 +9970,13 @@
         <v>0.208269148124244</v>
       </c>
       <c r="AW49" t="n">
-        <v>-0.2654902434403713</v>
+        <v>-0.2654899651378101</v>
       </c>
       <c r="AX49" t="n">
         <v>0.03450408380073022</v>
       </c>
       <c r="AY49" t="n">
-        <v>6.500327325998982</v>
+        <v>6.500329139686472</v>
       </c>
       <c r="AZ49" t="inlineStr"/>
       <c r="BA49" t="n">
@@ -10118,16 +10118,16 @@
         <v>1002.329603271484</v>
       </c>
       <c r="AG50" t="n">
-        <v>893.2902505493164</v>
+        <v>893.2902514648438</v>
       </c>
       <c r="AH50" t="n">
         <v>-0.04495485675885991</v>
       </c>
       <c r="AI50" t="n">
-        <v>0.07162259852560804</v>
+        <v>0.07162259742730903</v>
       </c>
       <c r="AJ50" t="n">
-        <v>0.122064863749622</v>
+        <v>0.122064862599625</v>
       </c>
       <c r="AK50" t="n">
         <v>1174.859985351562</v>
@@ -10167,10 +10167,10 @@
       </c>
       <c r="AW50" t="inlineStr"/>
       <c r="AX50" t="n">
-        <v>0.4112927267356079</v>
+        <v>0.4112925997426113</v>
       </c>
       <c r="AY50" t="n">
-        <v>6.324306944541086</v>
+        <v>6.324307799644687</v>
       </c>
       <c r="AZ50" t="inlineStr"/>
       <c r="BA50" t="n">
@@ -10312,28 +10312,28 @@
         <v>67.84656311035157</v>
       </c>
       <c r="AG51" t="n">
-        <v>62.96072395324707</v>
+        <v>62.96072414398193</v>
       </c>
       <c r="AH51" t="n">
         <v>-0.05138893320696514</v>
       </c>
       <c r="AI51" t="n">
-        <v>0.02222459605362159</v>
+        <v>0.02222459295686763</v>
       </c>
       <c r="AJ51" t="n">
-        <v>0.07760138146970141</v>
+        <v>0.07760137820518764</v>
       </c>
       <c r="AK51" t="n">
         <v>70.97299957275391</v>
       </c>
       <c r="AL51" t="n">
-        <v>55.35892868041992</v>
+        <v>55.35893249511719</v>
       </c>
       <c r="AM51" t="n">
         <v>-0.0931762642443118</v>
       </c>
       <c r="AN51" t="n">
-        <v>0.1625947637443219</v>
+        <v>0.1625946836317389</v>
       </c>
       <c r="AO51" t="n">
         <v>37.09052042422923</v>
@@ -10357,16 +10357,16 @@
         <v>0.03877805391089284</v>
       </c>
       <c r="AV51" t="n">
-        <v>0.1183147131905433</v>
+        <v>0.1183147873168129</v>
       </c>
       <c r="AW51" t="n">
-        <v>0.0283558119979237</v>
+        <v>0.02835556127690841</v>
       </c>
       <c r="AX51" t="n">
         <v>0.120204340034672</v>
       </c>
       <c r="AY51" t="n">
-        <v>174.9186635232768</v>
+        <v>174.9187495056376</v>
       </c>
       <c r="AZ51" t="inlineStr"/>
       <c r="BA51" t="n">
@@ -10508,16 +10508,16 @@
         <v>109.265920715332</v>
       </c>
       <c r="AG52" t="n">
-        <v>104.7508229446411</v>
+        <v>104.7508230209351</v>
       </c>
       <c r="AH52" t="n">
         <v>-0.03602146816235141</v>
       </c>
       <c r="AI52" t="n">
-        <v>0.005529110608702981</v>
+        <v>0.005529109876338367</v>
       </c>
       <c r="AJ52" t="n">
-        <v>0.04310322003939837</v>
+        <v>0.0431032192796672</v>
       </c>
       <c r="AK52" t="n">
         <v>116.6635665893555</v>
@@ -10556,13 +10556,13 @@
         <v>0.2013501666171391</v>
       </c>
       <c r="AW52" t="n">
-        <v>1.229217906321854</v>
+        <v>1.229218086297221</v>
       </c>
       <c r="AX52" t="n">
         <v>0.1425278409052821</v>
       </c>
       <c r="AY52" t="n">
-        <v>196.1452079662031</v>
+        <v>196.1451859723959</v>
       </c>
       <c r="AZ52" t="inlineStr"/>
       <c r="BA52" t="n">
@@ -10756,7 +10756,7 @@
         <v>-0.2190755155207131</v>
       </c>
       <c r="AY53" t="n">
-        <v>6.043039953472564</v>
+        <v>6.043040618005776</v>
       </c>
       <c r="AZ53" t="inlineStr"/>
       <c r="BA53" t="n">
@@ -10898,16 +10898,16 @@
         <v>123.5100679016113</v>
       </c>
       <c r="AG54" t="n">
-        <v>122.3461171340942</v>
+        <v>122.3461167907715</v>
       </c>
       <c r="AH54" t="n">
         <v>-0.03311527393802571</v>
       </c>
       <c r="AI54" t="n">
-        <v>-0.02391672930610322</v>
+        <v>-0.02391672656705757</v>
       </c>
       <c r="AJ54" t="n">
-        <v>0.009513589763060271</v>
+        <v>0.009513592595916665</v>
       </c>
       <c r="AK54" t="n">
         <v>131.1634063720703</v>
@@ -10940,19 +10940,19 @@
         <v>-0.03600892906742037</v>
       </c>
       <c r="AU54" t="n">
-        <v>-0.08741285813200106</v>
+        <v>-0.08741275171972063</v>
       </c>
       <c r="AV54" t="n">
-        <v>0.01229280570979929</v>
+        <v>0.01229274024237026</v>
       </c>
       <c r="AW54" t="n">
-        <v>0.370088932347046</v>
+        <v>0.3700892921228054</v>
       </c>
       <c r="AX54" t="n">
         <v>0.04347649280678301</v>
       </c>
       <c r="AY54" t="n">
-        <v>161.7225399053083</v>
+        <v>161.7225795531758</v>
       </c>
       <c r="AZ54" t="inlineStr"/>
       <c r="BA54" t="n">
@@ -11092,16 +11092,16 @@
         <v>148.8540002441406</v>
       </c>
       <c r="AG55" t="n">
-        <v>157.0050724029541</v>
+        <v>157.0050727081299</v>
       </c>
       <c r="AH55" t="n">
         <v>-0.00318429710018342</v>
       </c>
       <c r="AI55" t="n">
-        <v>-0.05493496094193273</v>
+        <v>-0.05493496277888588</v>
       </c>
       <c r="AJ55" t="n">
-        <v>-0.0519159797455061</v>
+        <v>-0.05191598158832733</v>
       </c>
       <c r="AK55" t="n">
         <v>217.0162200927734</v>
@@ -11137,16 +11137,16 @@
         <v>-0.06391631742452597</v>
       </c>
       <c r="AV55" t="n">
-        <v>-0.2690107178633612</v>
+        <v>-0.2690107728132318</v>
       </c>
       <c r="AW55" t="n">
-        <v>7.517854636257788</v>
+        <v>7.517857434185869</v>
       </c>
       <c r="AX55" t="n">
-        <v>-0.09949466780026628</v>
+        <v>-0.09949475119089068</v>
       </c>
       <c r="AY55" t="n">
-        <v>12.08738809441496</v>
+        <v>12.08738919527145</v>
       </c>
       <c r="AZ55" t="inlineStr"/>
       <c r="BA55" t="n">
@@ -11261,10 +11261,10 @@
         </is>
       </c>
       <c r="Z56" t="n">
-        <v>1.160227417945862</v>
+        <v>1.160092830657959</v>
       </c>
       <c r="AA56" t="n">
-        <v>142410275204.6982</v>
+        <v>142393755501.3945</v>
       </c>
       <c r="AB56" t="inlineStr">
         <is>
@@ -11525,16 +11525,16 @@
         <v>-0.1172077287486526</v>
       </c>
       <c r="AV57" t="n">
-        <v>0.02861186966113949</v>
+        <v>0.02861196317624026</v>
       </c>
       <c r="AW57" t="n">
-        <v>0.450988677832161</v>
+        <v>0.4509889569567094</v>
       </c>
       <c r="AX57" t="n">
         <v>0.009956801965402162</v>
       </c>
       <c r="AY57" t="n">
-        <v>176.6978896332866</v>
+        <v>176.6978242217564</v>
       </c>
       <c r="AZ57" t="inlineStr"/>
       <c r="BA57" t="n">
@@ -11724,13 +11724,13 @@
         <v>-0.0225949006443551</v>
       </c>
       <c r="AW58" t="n">
-        <v>0.5791290714273325</v>
+        <v>0.5791289623013243</v>
       </c>
       <c r="AX58" t="n">
         <v>0.02447311198179936</v>
       </c>
       <c r="AY58" t="n">
-        <v>323.0878071113752</v>
+        <v>323.0879148396873</v>
       </c>
       <c r="AZ58" t="inlineStr"/>
       <c r="BA58" t="n">
@@ -11922,7 +11922,7 @@
         <v>-0.4410642291427752</v>
       </c>
       <c r="AY59" t="n">
-        <v>-0.9299773823965434</v>
+        <v>-0.9299773902559232</v>
       </c>
       <c r="AZ59" t="inlineStr"/>
       <c r="BA59" t="n">
@@ -12444,16 +12444,16 @@
         <v>167.8812966918945</v>
       </c>
       <c r="AG62" t="n">
-        <v>191.8257102203369</v>
+        <v>191.8257099914551</v>
       </c>
       <c r="AH62" t="n">
         <v>-0.105796785733098</v>
       </c>
       <c r="AI62" t="n">
-        <v>-0.2174146263044976</v>
+        <v>-0.2174146253707356</v>
       </c>
       <c r="AJ62" t="n">
-        <v>-0.1248237970861105</v>
+        <v>-0.1248237960418713</v>
       </c>
       <c r="AK62" t="n">
         <v>237.7264404296875</v>
@@ -12492,13 +12492,13 @@
         <v>-0.112402644785095</v>
       </c>
       <c r="AW62" t="n">
-        <v>1.759188523620641</v>
+        <v>1.759188717077582</v>
       </c>
       <c r="AX62" t="n">
         <v>-0.1709335309286669</v>
       </c>
       <c r="AY62" t="n">
-        <v>9.611075241780931</v>
+        <v>9.611075957067982</v>
       </c>
       <c r="AZ62" t="inlineStr"/>
       <c r="BA62" t="n">
@@ -12690,7 +12690,7 @@
         <v>-0.01907464793006219</v>
       </c>
       <c r="AY63" t="n">
-        <v>15.1577955620556</v>
+        <v>15.15779813735503</v>
       </c>
       <c r="AZ63" t="inlineStr"/>
       <c r="BA63" t="n">
@@ -12801,7 +12801,7 @@
         </is>
       </c>
       <c r="X64" t="n">
-        <v>171696865280</v>
+        <v>171666178048</v>
       </c>
       <c r="Y64" t="inlineStr">
         <is>
@@ -12812,7 +12812,7 @@
         <v>1</v>
       </c>
       <c r="AA64" t="n">
-        <v>171696865280</v>
+        <v>171666178048</v>
       </c>
       <c r="AB64" t="inlineStr">
         <is>
@@ -12832,28 +12832,28 @@
         <v>85.63172836303711</v>
       </c>
       <c r="AG64" t="n">
-        <v>86.55546867370606</v>
+        <v>86.55546863555908</v>
       </c>
       <c r="AH64" t="n">
         <v>-0.03879088823666887</v>
       </c>
       <c r="AI64" t="n">
-        <v>-0.04904913785536469</v>
+        <v>-0.04904913743625883</v>
       </c>
       <c r="AJ64" t="n">
-        <v>-0.0106722350976024</v>
+        <v>-0.01067223466158296</v>
       </c>
       <c r="AK64" t="n">
         <v>96.44304656982422</v>
       </c>
       <c r="AL64" t="n">
-        <v>67.87922668457031</v>
+        <v>67.87921905517578</v>
       </c>
       <c r="AM64" t="n">
         <v>-0.1465429547686283</v>
       </c>
       <c r="AN64" t="n">
-        <v>0.212594803725183</v>
+        <v>0.212594940016736</v>
       </c>
       <c r="AO64" t="n">
         <v>44.95100260838581</v>
@@ -12880,10 +12880,10 @@
         <v>0.1872616281865767</v>
       </c>
       <c r="AW64" t="n">
-        <v>0.09870477819140677</v>
+        <v>0.09870500197569698</v>
       </c>
       <c r="AX64" t="n">
-        <v>0.03924345910238802</v>
+        <v>0.03924355921115819</v>
       </c>
       <c r="AY64" t="n">
         <v>237.6419604019922</v>
@@ -13028,25 +13028,25 @@
         <v>124.7768704223633</v>
       </c>
       <c r="AG65" t="n">
-        <v>144.878759727478</v>
+        <v>144.8787600326538</v>
       </c>
       <c r="AH65" t="n">
         <v>-0.09069686793380538</v>
       </c>
       <c r="AI65" t="n">
-        <v>-0.2168624351982662</v>
+        <v>-0.2168624368478842</v>
       </c>
       <c r="AJ65" t="n">
-        <v>-0.1387497335215121</v>
+        <v>-0.1387497353356684</v>
       </c>
       <c r="AK65" t="n">
-        <v>182.8191833496094</v>
+        <v>182.8191986083984</v>
       </c>
       <c r="AL65" t="n">
         <v>109.5100021362305</v>
       </c>
       <c r="AM65" t="n">
-        <v>-0.3793867962559462</v>
+        <v>-0.3793868480546961</v>
       </c>
       <c r="AN65" t="n">
         <v>0.0360697367472278</v>
@@ -13070,10 +13070,10 @@
         <v>-0.09251021239810941</v>
       </c>
       <c r="AU65" t="n">
-        <v>-0.2528851336116935</v>
+        <v>-0.2528852086792028</v>
       </c>
       <c r="AV65" t="n">
-        <v>-0.2726567418387896</v>
+        <v>-0.2726565995449136</v>
       </c>
       <c r="AW65" t="n">
         <v>1.848101789458746</v>
@@ -13082,7 +13082,7 @@
         <v>-0.3104960057120867</v>
       </c>
       <c r="AY65" t="n">
-        <v>14.89347478983514</v>
+        <v>14.89346948178655</v>
       </c>
       <c r="AZ65" t="inlineStr"/>
       <c r="BA65" t="n">
@@ -13189,7 +13189,7 @@
         </is>
       </c>
       <c r="X66" t="n">
-        <v>6604485632</v>
+        <v>6519808000</v>
       </c>
       <c r="Y66" t="inlineStr">
         <is>
@@ -13200,7 +13200,7 @@
         <v>1</v>
       </c>
       <c r="AA66" t="n">
-        <v>6604485632</v>
+        <v>6519808000</v>
       </c>
       <c r="AB66" t="inlineStr">
         <is>
@@ -13606,16 +13606,16 @@
         <v>181.4109027099609</v>
       </c>
       <c r="AG68" t="n">
-        <v>131.7051400756836</v>
+        <v>131.7051403045654</v>
       </c>
       <c r="AH68" t="n">
         <v>0.09850067334654633</v>
       </c>
       <c r="AI68" t="n">
-        <v>0.5130768523140536</v>
+        <v>0.5130768496845757</v>
       </c>
       <c r="AJ68" t="n">
-        <v>0.3774018432820025</v>
+        <v>0.3774018408883053</v>
       </c>
       <c r="AK68" t="n">
         <v>207.0800018310547</v>
@@ -13651,16 +13651,16 @@
         <v>1.036378315962156</v>
       </c>
       <c r="AV68" t="n">
-        <v>0.6209733872697376</v>
+        <v>0.6209734878651461</v>
       </c>
       <c r="AW68" t="n">
-        <v>1.444390914961116</v>
+        <v>1.444391143714604</v>
       </c>
       <c r="AX68" t="n">
         <v>0.8870019371368951</v>
       </c>
       <c r="AY68" t="n">
-        <v>211.5167853794182</v>
+        <v>211.5167988877866</v>
       </c>
       <c r="AZ68" t="inlineStr"/>
       <c r="BA68" t="n">
@@ -13846,7 +13846,7 @@
         <v>9.579347526230009</v>
       </c>
       <c r="AW69" t="n">
-        <v>6.058741742898738</v>
+        <v>6.058743285053041</v>
       </c>
       <c r="AX69" t="n">
         <v>1.389297060726459</v>
@@ -13967,10 +13967,10 @@
         </is>
       </c>
       <c r="Z70" t="n">
-        <v>0.0007456843159161508</v>
+        <v>0.0007449344266206026</v>
       </c>
       <c r="AA70" t="n">
-        <v>959141726498.1094</v>
+        <v>958177176086.8125</v>
       </c>
       <c r="AB70" t="inlineStr">
         <is>
@@ -13990,16 +13990,16 @@
         <v>1756381.4375</v>
       </c>
       <c r="AG70" t="n">
-        <v>1336251.39546875</v>
+        <v>1336251.3965625</v>
       </c>
       <c r="AH70" t="n">
         <v>0.03166656246331456</v>
       </c>
       <c r="AI70" t="n">
-        <v>0.3560322602053185</v>
+        <v>0.3560322590953775</v>
       </c>
       <c r="AJ70" t="n">
-        <v>0.3144094318299069</v>
+        <v>0.314409430754035</v>
       </c>
       <c r="AK70" t="n">
         <v>2918367.25</v>
@@ -14035,16 +14035,16 @@
         <v>0.9491354442737323</v>
       </c>
       <c r="AV70" t="n">
-        <v>5.755916757653973</v>
+        <v>5.755915970498794</v>
       </c>
       <c r="AW70" t="n">
-        <v>14.47712080550214</v>
+        <v>14.47711873992167</v>
       </c>
       <c r="AX70" t="n">
         <v>1.682482754741024</v>
       </c>
       <c r="AY70" t="n">
-        <v>-8.918744914984863</v>
+        <v>-8.918742211372678</v>
       </c>
       <c r="AZ70" t="inlineStr"/>
       <c r="BA70" t="n">
@@ -14163,10 +14163,10 @@
         </is>
       </c>
       <c r="Z71" t="n">
-        <v>0.0007456843159161508</v>
+        <v>0.0007449344266206026</v>
       </c>
       <c r="AA71" t="n">
-        <v>1270663355118.422</v>
+        <v>1269385526380.562</v>
       </c>
       <c r="AB71" t="inlineStr">
         <is>
@@ -14186,28 +14186,28 @@
         <v>259460</v>
       </c>
       <c r="AG71" t="n">
-        <v>215571.015390625</v>
+        <v>215571.0155859375</v>
       </c>
       <c r="AH71" t="n">
         <v>0.0001541663454867059</v>
       </c>
       <c r="AI71" t="n">
-        <v>0.2037796432408763</v>
+        <v>0.2037796421502229</v>
       </c>
       <c r="AJ71" t="n">
-        <v>0.2035940895386426</v>
+        <v>0.2035940884481575</v>
       </c>
       <c r="AK71" t="n">
         <v>362100.65625</v>
       </c>
       <c r="AL71" t="n">
-        <v>66762.203125</v>
+        <v>66762.1953125</v>
       </c>
       <c r="AM71" t="n">
         <v>-0.2833484404931951</v>
       </c>
       <c r="AN71" t="n">
-        <v>2.886929847328941</v>
+        <v>2.886930302176768</v>
       </c>
       <c r="AO71" t="n">
         <v>51.96850393700787</v>
@@ -14228,19 +14228,19 @@
         <v>-0.2291211015101948</v>
       </c>
       <c r="AU71" t="n">
-        <v>0.3854384314514545</v>
+        <v>0.3854385470246606</v>
       </c>
       <c r="AV71" t="n">
-        <v>2.769819899623551</v>
+        <v>2.769820327475903</v>
       </c>
       <c r="AW71" t="n">
-        <v>2.558768809131345</v>
+        <v>2.55876804655712</v>
       </c>
       <c r="AX71" t="n">
         <v>1.0258668851272</v>
       </c>
       <c r="AY71" t="n">
-        <v>59.78044434583563</v>
+        <v>59.7804512970467</v>
       </c>
       <c r="AZ71" t="inlineStr"/>
       <c r="BA71" t="n">
@@ -14426,13 +14426,13 @@
         <v>7.492507565916174</v>
       </c>
       <c r="AW72" t="n">
-        <v>4.333660455963548</v>
+        <v>4.333661088734792</v>
       </c>
       <c r="AX72" t="n">
         <v>0.8986552642408132</v>
       </c>
       <c r="AY72" t="n">
-        <v>3.505365126646732</v>
+        <v>3.50536557814489</v>
       </c>
       <c r="AZ72" t="inlineStr"/>
       <c r="BA72" t="n">
@@ -14779,13 +14779,13 @@
         <v>433.3299865722656</v>
       </c>
       <c r="AL74" t="n">
-        <v>114.9438400268555</v>
+        <v>114.94384765625</v>
       </c>
       <c r="AM74" t="n">
         <v>-0.3117946819704582</v>
       </c>
       <c r="AN74" t="n">
-        <v>1.594484412135762</v>
+        <v>1.594484239926934</v>
       </c>
       <c r="AO74" t="n">
         <v>42.17106145701388</v>
@@ -14809,7 +14809,7 @@
         <v>0.4063622593446763</v>
       </c>
       <c r="AV74" t="n">
-        <v>1.594484412135762</v>
+        <v>1.594484239926934</v>
       </c>
       <c r="AW74" t="n">
         <v>4.144068438445124</v>
@@ -14818,7 +14818,7 @@
         <v>0.6145445719687945</v>
       </c>
       <c r="AY74" t="n">
-        <v>1580.800987088059</v>
+        <v>1580.801237132436</v>
       </c>
       <c r="AZ74" t="inlineStr"/>
       <c r="BA74" t="n">
@@ -14960,16 +14960,16 @@
         <v>928.6070019531249</v>
       </c>
       <c r="AG75" t="n">
-        <v>621.9325052642822</v>
+        <v>621.9325054168701</v>
       </c>
       <c r="AH75" t="n">
         <v>0.05023977604559904</v>
       </c>
       <c r="AI75" t="n">
-        <v>0.5681122975735138</v>
+        <v>0.5681122971887858</v>
       </c>
       <c r="AJ75" t="n">
-        <v>0.4930993220213267</v>
+        <v>0.4930993216550026</v>
       </c>
       <c r="AK75" t="n">
         <v>1213.373413085938</v>
@@ -15002,7 +15002,7 @@
         <v>-0.006316142964417515</v>
       </c>
       <c r="AU75" t="n">
-        <v>1.289957921719005</v>
+        <v>1.289957757628058</v>
       </c>
       <c r="AV75" t="n">
         <v>5.4875162188819</v>
@@ -15011,7 +15011,7 @@
         <v>12.55000890936919</v>
       </c>
       <c r="AX75" t="n">
-        <v>2.093715194600453</v>
+        <v>2.093715494095987</v>
       </c>
       <c r="AY75" t="n">
         <v>721.0154401002217</v>
@@ -15350,28 +15350,28 @@
         <v>848.2073986816406</v>
       </c>
       <c r="AG77" t="n">
-        <v>605.2932033538818</v>
+        <v>605.293203125</v>
       </c>
       <c r="AH77" t="n">
         <v>-0.02126533651972351</v>
       </c>
       <c r="AI77" t="n">
-        <v>0.3715171066026348</v>
+        <v>0.3715171071212517</v>
       </c>
       <c r="AJ77" t="n">
-        <v>0.4013165751437326</v>
+        <v>0.4013165756736179</v>
       </c>
       <c r="AK77" t="n">
         <v>1093.260498046875</v>
       </c>
       <c r="AL77" t="n">
-        <v>194.3849945068359</v>
+        <v>194.3850250244141</v>
       </c>
       <c r="AM77" t="n">
         <v>-0.2406476000978116</v>
       </c>
       <c r="AN77" t="n">
-        <v>3.270751376752806</v>
+        <v>3.270750706263972</v>
       </c>
       <c r="AO77" t="n">
         <v>47.05322685241872</v>
@@ -15398,13 +15398,13 @@
         <v>3.252957295731137</v>
       </c>
       <c r="AW77" t="n">
-        <v>9.669445383582952</v>
+        <v>9.669444337402275</v>
       </c>
       <c r="AX77" t="n">
         <v>1.894244516598677</v>
       </c>
       <c r="AY77" t="n">
-        <v>156.4856891850746</v>
+        <v>156.4857461680869</v>
       </c>
       <c r="AZ77" t="inlineStr"/>
       <c r="BA77" t="n">
@@ -15544,28 +15544,28 @@
         <v>494.6775927734375</v>
       </c>
       <c r="AG78" t="n">
-        <v>379.0106123352051</v>
+        <v>379.0106120300293</v>
       </c>
       <c r="AH78" t="n">
         <v>-0.09601728639326135</v>
       </c>
       <c r="AI78" t="n">
-        <v>0.1798614026149901</v>
+        <v>0.1798614035650032</v>
       </c>
       <c r="AJ78" t="n">
-        <v>0.3051813766521505</v>
+        <v>0.3051813777030703</v>
       </c>
       <c r="AK78" t="n">
         <v>745.990478515625</v>
       </c>
       <c r="AL78" t="n">
-        <v>95.97096252441406</v>
+        <v>95.97095489501953</v>
       </c>
       <c r="AM78" t="n">
         <v>-0.4005553615569171</v>
       </c>
       <c r="AN78" t="n">
-        <v>3.659534310307903</v>
+        <v>3.65953468072649</v>
       </c>
       <c r="AO78" t="n">
         <v>46.23351960205819</v>
@@ -15586,19 +15586,19 @@
         <v>-0.2053655687556025</v>
       </c>
       <c r="AU78" t="n">
-        <v>0.6432487291428597</v>
+        <v>0.6432485448645322</v>
       </c>
       <c r="AV78" t="n">
-        <v>3.659534310307903</v>
+        <v>3.65953468072649</v>
       </c>
       <c r="AW78" t="n">
-        <v>8.68113573619271</v>
+        <v>8.681136535714616</v>
       </c>
       <c r="AX78" t="n">
-        <v>1.38494598664461</v>
+        <v>1.384945792558361</v>
       </c>
       <c r="AY78" t="n">
-        <v>657.2740277355766</v>
+        <v>657.2739699777102</v>
       </c>
       <c r="AZ78" t="inlineStr"/>
       <c r="BA78" t="n">
@@ -15709,7 +15709,7 @@
         </is>
       </c>
       <c r="X79" t="n">
-        <v>9432905728</v>
+        <v>9404672000</v>
       </c>
       <c r="Y79" t="inlineStr">
         <is>
@@ -15720,7 +15720,7 @@
         <v>1</v>
       </c>
       <c r="AA79" t="n">
-        <v>9432905728</v>
+        <v>9404672000</v>
       </c>
       <c r="AB79" t="inlineStr">
         <is>
@@ -16246,28 +16246,28 @@
         <v>80.27049957275391</v>
       </c>
       <c r="AG82" t="n">
-        <v>73.0320651435852</v>
+        <v>73.03206558227539</v>
       </c>
       <c r="AH82" t="n">
         <v>0.04546500414992005</v>
       </c>
       <c r="AI82" t="n">
-        <v>0.1490842824169605</v>
+        <v>0.1490842755146224</v>
       </c>
       <c r="AJ82" t="n">
-        <v>0.09911310073099444</v>
+        <v>0.09911309412882408</v>
       </c>
       <c r="AK82" t="n">
         <v>88.16000366210938</v>
       </c>
       <c r="AL82" t="n">
-        <v>58.88565826416016</v>
+        <v>58.88565444946289</v>
       </c>
       <c r="AM82" t="n">
         <v>-0.04809443417691683</v>
       </c>
       <c r="AN82" t="n">
-        <v>0.4251347550957398</v>
+        <v>0.4251348474180161</v>
       </c>
       <c r="AO82" t="n">
         <v>64.498009818745</v>
@@ -16294,13 +16294,13 @@
         <v>0.4144474977009491</v>
       </c>
       <c r="AW82" t="n">
-        <v>3.558486571925111</v>
+        <v>3.558487044212144</v>
       </c>
       <c r="AX82" t="n">
-        <v>0.2055359538563837</v>
+        <v>0.2055360859813806</v>
       </c>
       <c r="AY82" t="n">
-        <v>1340.28236987739</v>
+        <v>1340.282849043941</v>
       </c>
       <c r="AZ82" t="inlineStr"/>
       <c r="BA82" t="n">
@@ -17195,10 +17195,10 @@
         </is>
       </c>
       <c r="Z87" t="n">
-        <v>1.160227417945862</v>
+        <v>1.160092830657959</v>
       </c>
       <c r="AA87" t="n">
-        <v>7203788995.908875</v>
+        <v>7202953350.751221</v>
       </c>
       <c r="AB87" t="inlineStr">
         <is>
@@ -17209,7 +17209,7 @@
         <v>37055</v>
       </c>
       <c r="AD87" t="n">
-        <v>25.2</v>
+        <v>25.3</v>
       </c>
       <c r="AE87" t="n">
         <v>142.1999969482422</v>
@@ -17266,13 +17266,13 @@
         <v>0.08141723482576002</v>
       </c>
       <c r="AW87" t="n">
-        <v>1.041217429777988</v>
+        <v>1.041217206230922</v>
       </c>
       <c r="AX87" t="n">
         <v>0.1286185580544279</v>
       </c>
       <c r="AY87" t="n">
-        <v>7.80497333721339</v>
+        <v>7.804974377101559</v>
       </c>
       <c r="AZ87" t="inlineStr"/>
       <c r="BA87" t="n">
@@ -17458,7 +17458,7 @@
         <v>1.409090993536689</v>
       </c>
       <c r="AW88" t="n">
-        <v>1.051402790332227</v>
+        <v>1.051402970624388</v>
       </c>
       <c r="AX88" t="n">
         <v>0.7096773768243965</v>
@@ -17571,7 +17571,7 @@
         </is>
       </c>
       <c r="X89" t="n">
-        <v>37188722688</v>
+        <v>37188132864</v>
       </c>
       <c r="Y89" t="inlineStr">
         <is>
@@ -17579,10 +17579,10 @@
         </is>
       </c>
       <c r="Z89" t="n">
-        <v>1.160227417945862</v>
+        <v>1.160092830657959</v>
       </c>
       <c r="AA89" t="n">
-        <v>43147375701.00293</v>
+        <v>43141686321.08203</v>
       </c>
       <c r="AB89" t="inlineStr">
         <is>
@@ -17771,10 +17771,10 @@
         </is>
       </c>
       <c r="Z90" t="n">
-        <v>0.1490868479013443</v>
+        <v>0.1490846127271652</v>
       </c>
       <c r="AA90" t="n">
-        <v>21890013975.73853</v>
+        <v>21889685791.22925</v>
       </c>
       <c r="AB90" t="inlineStr">
         <is>
@@ -17842,13 +17842,13 @@
         <v>1.581283699222637</v>
       </c>
       <c r="AW90" t="n">
-        <v>6.915992228703978</v>
+        <v>6.915991554820075</v>
       </c>
       <c r="AX90" t="n">
         <v>1.504023662647851</v>
       </c>
       <c r="AY90" t="n">
-        <v>19.36990945146228</v>
+        <v>19.36990722034421</v>
       </c>
       <c r="AZ90" t="inlineStr"/>
       <c r="BA90" t="n">
@@ -17955,7 +17955,7 @@
         </is>
       </c>
       <c r="X91" t="n">
-        <v>1083174289408</v>
+        <v>1090744287232</v>
       </c>
       <c r="Y91" t="inlineStr">
         <is>
@@ -17963,10 +17963,10 @@
         </is>
       </c>
       <c r="Z91" t="n">
-        <v>0.1490868479013443</v>
+        <v>0.1490846127271652</v>
       </c>
       <c r="AA91" t="n">
-        <v>161487040535.6172</v>
+        <v>162613189646.3506</v>
       </c>
       <c r="AB91" t="inlineStr">
         <is>
@@ -18155,10 +18155,10 @@
         </is>
       </c>
       <c r="Z92" t="n">
-        <v>0.1490868479013443</v>
+        <v>0.1490846127271652</v>
       </c>
       <c r="AA92" t="n">
-        <v>87927037973.69629</v>
+        <v>87925719733.70605</v>
       </c>
       <c r="AB92" t="inlineStr">
         <is>
@@ -18232,7 +18232,7 @@
         <v>0.3906082408166636</v>
       </c>
       <c r="AY92" t="n">
-        <v>228.3949700793907</v>
+        <v>228.3949552495158</v>
       </c>
       <c r="AZ92" t="inlineStr"/>
       <c r="BA92" t="n">
@@ -18537,7 +18537,7 @@
         </is>
       </c>
       <c r="X94" t="n">
-        <v>143335014400</v>
+        <v>143043723264</v>
       </c>
       <c r="Y94" t="inlineStr">
         <is>
@@ -18548,7 +18548,7 @@
         <v>1</v>
       </c>
       <c r="AA94" t="n">
-        <v>143335014400</v>
+        <v>143043723264</v>
       </c>
       <c r="AB94" t="inlineStr">
         <is>
@@ -18616,13 +18616,13 @@
         <v>1.224077457323134</v>
       </c>
       <c r="AW94" t="n">
-        <v>3.775291003593885</v>
+        <v>3.775290480828999</v>
       </c>
       <c r="AX94" t="n">
         <v>0.8449372876054011</v>
       </c>
       <c r="AY94" t="n">
-        <v>216.4702649445689</v>
+        <v>216.4702988256008</v>
       </c>
       <c r="AZ94" t="inlineStr"/>
       <c r="BA94" t="n">
@@ -18764,28 +18764,28 @@
         <v>216.8398794555664</v>
       </c>
       <c r="AG95" t="n">
-        <v>154.7597800064087</v>
+        <v>154.7597797775269</v>
       </c>
       <c r="AH95" t="n">
         <v>0.08882188413084724</v>
       </c>
       <c r="AI95" t="n">
-        <v>0.5255902153242824</v>
+        <v>0.5255902175805527</v>
       </c>
       <c r="AJ95" t="n">
-        <v>0.4011384575927086</v>
+        <v>0.4011384596649212</v>
       </c>
       <c r="AK95" t="n">
         <v>316.3519592285156</v>
       </c>
       <c r="AL95" t="n">
-        <v>66.44841766357422</v>
+        <v>66.44842529296875</v>
       </c>
       <c r="AM95" t="n">
         <v>-0.2536793302014302</v>
       </c>
       <c r="AN95" t="n">
-        <v>2.553132104648163</v>
+        <v>2.553131696688959</v>
       </c>
       <c r="AO95" t="n">
         <v>49.56449814743989</v>
@@ -18809,16 +18809,16 @@
         <v>1.689238258735586</v>
       </c>
       <c r="AV95" t="n">
-        <v>2.553132104648163</v>
+        <v>2.553131696688959</v>
       </c>
       <c r="AW95" t="n">
-        <v>2.910343169222694</v>
+        <v>2.910344157443346</v>
       </c>
       <c r="AX95" t="n">
         <v>1.645110953951491</v>
       </c>
       <c r="AY95" t="n">
-        <v>18.46524987496561</v>
+        <v>18.46525905777374</v>
       </c>
       <c r="AZ95" t="inlineStr"/>
       <c r="BA95" t="n">
@@ -18924,7 +18924,9 @@
           <t>DKK</t>
         </is>
       </c>
-      <c r="X96" t="inlineStr"/>
+      <c r="X96" t="n">
+        <v>49414942720</v>
+      </c>
       <c r="Y96" t="inlineStr">
         <is>
           <t>DKK</t>
@@ -18933,10 +18935,12 @@
       <c r="Z96" t="n">
         <v>0.1551782935857773</v>
       </c>
-      <c r="AA96" t="inlineStr"/>
+      <c r="AA96" t="n">
+        <v>7668126488.928528</v>
+      </c>
       <c r="AB96" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Mid cap</t>
         </is>
       </c>
       <c r="AC96" s="2" t="n">
@@ -19006,7 +19010,7 @@
         <v>0.1219660194174756</v>
       </c>
       <c r="AY96" t="n">
-        <v>26.37210534198059</v>
+        <v>26.37210225047868</v>
       </c>
       <c r="AZ96" t="inlineStr"/>
       <c r="BA96" t="n">
@@ -19117,7 +19121,7 @@
         </is>
       </c>
       <c r="X97" t="n">
-        <v>61365223424</v>
+        <v>61455826944</v>
       </c>
       <c r="Y97" t="inlineStr">
         <is>
@@ -19128,7 +19132,7 @@
         <v>1</v>
       </c>
       <c r="AA97" t="n">
-        <v>61365223424</v>
+        <v>61455826944</v>
       </c>
       <c r="AB97" t="inlineStr">
         <is>
@@ -19148,16 +19152,16 @@
         <v>205.5617034912109</v>
       </c>
       <c r="AG97" t="n">
-        <v>214.3561728668213</v>
+        <v>214.3561724090576</v>
       </c>
       <c r="AH97" t="n">
         <v>0.03112594960047987</v>
       </c>
       <c r="AI97" t="n">
-        <v>-0.01117843316993172</v>
+        <v>-0.01117843105827532</v>
       </c>
       <c r="AJ97" t="n">
-        <v>-0.04102736701253906</v>
+        <v>-0.04102736496462589</v>
       </c>
       <c r="AK97" t="n">
         <v>246.3216247558594</v>
@@ -19196,13 +19200,13 @@
         <v>0.008779446100566801</v>
       </c>
       <c r="AW97" t="n">
-        <v>0.5305453799018649</v>
+        <v>0.5305457171803649</v>
       </c>
       <c r="AX97" t="n">
         <v>-0.08127626505466301</v>
       </c>
       <c r="AY97" t="n">
-        <v>6.962670461796258</v>
+        <v>6.962673885097205</v>
       </c>
       <c r="AZ97" t="inlineStr"/>
       <c r="BA97" t="n">
@@ -19344,16 +19348,16 @@
         <v>383.0855993652344</v>
       </c>
       <c r="AG98" t="n">
-        <v>369.4377291870117</v>
+        <v>369.437728729248</v>
       </c>
       <c r="AH98" t="n">
         <v>-0.05506761195360621</v>
       </c>
       <c r="AI98" t="n">
-        <v>-0.02015965984044532</v>
+        <v>-0.02015965862634261</v>
       </c>
       <c r="AJ98" t="n">
-        <v>0.03694227497623559</v>
+        <v>0.03694227626109226</v>
       </c>
       <c r="AK98" t="n">
         <v>480.8090515136719</v>
@@ -19389,16 +19393,16 @@
         <v>0.1277732642630893</v>
       </c>
       <c r="AV98" t="n">
-        <v>0.01393743323475483</v>
+        <v>0.01393734656336121</v>
       </c>
       <c r="AW98" t="n">
-        <v>6.989550400843566</v>
+        <v>6.989549055484776</v>
       </c>
       <c r="AX98" t="n">
         <v>0.0451742685812544</v>
       </c>
       <c r="AY98" t="n">
-        <v>317.7678861779656</v>
+        <v>317.7679865664864</v>
       </c>
       <c r="AZ98" t="inlineStr"/>
       <c r="BA98" t="n">
@@ -19930,16 +19934,16 @@
         <v>78.22238220214844</v>
       </c>
       <c r="AG101" t="n">
-        <v>77.04982259750366</v>
+        <v>77.04982248306274</v>
       </c>
       <c r="AH101" t="n">
         <v>-0.05142243358827003</v>
       </c>
       <c r="AI101" t="n">
-        <v>-0.03698679053615117</v>
+        <v>-0.03698678910580244</v>
       </c>
       <c r="AJ101" t="n">
-        <v>0.01521819992720874</v>
+        <v>0.01521820143509678</v>
       </c>
       <c r="AK101" t="n">
         <v>102.0957336425781</v>
@@ -19975,16 +19979,16 @@
         <v>0.2111894718443408</v>
       </c>
       <c r="AV101" t="n">
-        <v>0.1710775498521604</v>
+        <v>0.1710776203583959</v>
       </c>
       <c r="AW101" t="n">
-        <v>0.05534037577789719</v>
+        <v>0.05534049029526078</v>
       </c>
       <c r="AX101" t="n">
-        <v>0.1604306491015695</v>
+        <v>0.1604307875616626</v>
       </c>
       <c r="AY101" t="n">
-        <v>423.9102286367834</v>
+        <v>423.9101561196683</v>
       </c>
       <c r="AZ101" t="inlineStr"/>
       <c r="BA101" t="n">
@@ -20091,7 +20095,7 @@
         </is>
       </c>
       <c r="X102" t="n">
-        <v>45943218176</v>
+        <v>45949857792</v>
       </c>
       <c r="Y102" t="inlineStr">
         <is>
@@ -20102,7 +20106,7 @@
         <v>1</v>
       </c>
       <c r="AA102" t="n">
-        <v>45943218176</v>
+        <v>45949857792</v>
       </c>
       <c r="AB102" t="inlineStr">
         <is>
@@ -20122,16 +20126,16 @@
         <v>56.26079986572265</v>
       </c>
       <c r="AG102" t="n">
-        <v>45.81929414749145</v>
+        <v>45.81929413795471</v>
       </c>
       <c r="AH102" t="n">
         <v>-0.08444248136407873</v>
       </c>
       <c r="AI102" t="n">
-        <v>0.1241988616350893</v>
+        <v>0.1241988618690779</v>
       </c>
       <c r="AJ102" t="n">
-        <v>0.2278844733971717</v>
+        <v>0.2278844736527412</v>
       </c>
       <c r="AK102" t="n">
         <v>79.81999969482422</v>
@@ -20167,16 +20171,16 @@
         <v>0.5733219256251763</v>
       </c>
       <c r="AV102" t="n">
-        <v>0.9906641160446528</v>
+        <v>0.9906639693093913</v>
       </c>
       <c r="AW102" t="n">
-        <v>0.19678205393756</v>
+        <v>0.1967819478660771</v>
       </c>
       <c r="AX102" t="n">
         <v>0.8894807230605781</v>
       </c>
       <c r="AY102" t="n">
-        <v>22.52406792963226</v>
+        <v>22.5240628068805</v>
       </c>
       <c r="AZ102" t="inlineStr"/>
       <c r="BA102" t="n">
@@ -20477,7 +20481,7 @@
         </is>
       </c>
       <c r="X104" t="n">
-        <v>165213700096</v>
+        <v>165171167232</v>
       </c>
       <c r="Y104" t="inlineStr">
         <is>
@@ -20488,7 +20492,7 @@
         <v>1</v>
       </c>
       <c r="AA104" t="n">
-        <v>165213700096</v>
+        <v>165171167232</v>
       </c>
       <c r="AB104" t="inlineStr">
         <is>
@@ -20508,28 +20512,28 @@
         <v>415.2714404296875</v>
       </c>
       <c r="AG104" t="n">
-        <v>380.9242803955078</v>
+        <v>380.9242797851563</v>
       </c>
       <c r="AH104" t="n">
         <v>0.02431796098727834</v>
       </c>
       <c r="AI104" t="n">
-        <v>0.1166786078207784</v>
+        <v>0.1166786096100225</v>
       </c>
       <c r="AJ104" t="n">
-        <v>0.09016794623466251</v>
+        <v>0.09016794798142902</v>
       </c>
       <c r="AK104" t="n">
         <v>459.9599914550781</v>
       </c>
       <c r="AL104" t="n">
-        <v>313.2000122070312</v>
+        <v>313.2000427246094</v>
       </c>
       <c r="AM104" t="n">
         <v>-0.07520218493018394</v>
       </c>
       <c r="AN104" t="n">
-        <v>0.358141693928191</v>
+        <v>0.3581415615936137</v>
       </c>
       <c r="AO104" t="n">
         <v>52.78806215490184</v>
@@ -20556,13 +20560,13 @@
         <v>0.1944917302253835</v>
       </c>
       <c r="AW104" t="n">
-        <v>1.762786948235172</v>
+        <v>1.762787495853646</v>
       </c>
       <c r="AX104" t="n">
         <v>0.3104650208403865</v>
       </c>
       <c r="AY104" t="n">
-        <v>1233.591858710512</v>
+        <v>1233.592392660112</v>
       </c>
       <c r="AZ104" t="inlineStr"/>
       <c r="BA104" t="n">
@@ -20677,10 +20681,10 @@
         </is>
       </c>
       <c r="Z105" t="n">
-        <v>1.160227417945862</v>
+        <v>1.160092830657959</v>
       </c>
       <c r="AA105" t="n">
-        <v>190268901620.1797</v>
+        <v>190246830278.7812</v>
       </c>
       <c r="AB105" t="inlineStr">
         <is>
@@ -20748,13 +20752,13 @@
         <v>0.291634890681584</v>
       </c>
       <c r="AW105" t="n">
-        <v>1.298819148076014</v>
+        <v>1.298819563583454</v>
       </c>
       <c r="AX105" t="n">
         <v>0.2472272894666976</v>
       </c>
       <c r="AY105" t="n">
-        <v>14.64281869989337</v>
+        <v>14.64282350982918</v>
       </c>
       <c r="AZ105" t="inlineStr"/>
       <c r="BA105" t="n">
@@ -20861,7 +20865,7 @@
         </is>
       </c>
       <c r="X106" t="n">
-        <v>628541685760</v>
+        <v>628726824960</v>
       </c>
       <c r="Y106" t="inlineStr">
         <is>
@@ -20872,7 +20876,7 @@
         <v>0.03161855414509773</v>
       </c>
       <c r="AA106" t="n">
-        <v>19873579323.65356</v>
+        <v>19879433157.47314</v>
       </c>
       <c r="AB106" t="inlineStr">
         <is>
@@ -20940,7 +20944,7 @@
         <v>1.25855018110979</v>
       </c>
       <c r="AW106" t="n">
-        <v>5.20030992204815</v>
+        <v>5.200309392619952</v>
       </c>
       <c r="AX106" t="n">
         <v>0.7040558252684641</v>
@@ -21061,10 +21065,10 @@
         </is>
       </c>
       <c r="Z107" t="n">
-        <v>1.160227417945862</v>
+        <v>1.160092830657959</v>
       </c>
       <c r="AA107" t="n">
-        <v>43138203778.40039</v>
+        <v>43133199713.02344</v>
       </c>
       <c r="AB107" t="inlineStr">
         <is>
@@ -21132,13 +21136,13 @@
         <v>0.04725705494249</v>
       </c>
       <c r="AW107" t="n">
-        <v>0.7460674058115271</v>
+        <v>0.7460672418346221</v>
       </c>
       <c r="AX107" t="n">
         <v>0.1279728663777335</v>
       </c>
       <c r="AY107" t="n">
-        <v>9.475951386231095</v>
+        <v>9.475949910566657</v>
       </c>
       <c r="AZ107" t="inlineStr"/>
       <c r="BA107" t="n">
@@ -21330,7 +21334,7 @@
         <v>0.6366542354821523</v>
       </c>
       <c r="AY108" t="n">
-        <v>64.58186176027263</v>
+        <v>64.58188707963257</v>
       </c>
       <c r="AZ108" t="inlineStr"/>
       <c r="BA108" t="n">
@@ -21520,13 +21524,13 @@
         <v>0.5449460152910517</v>
       </c>
       <c r="AW109" t="n">
-        <v>1.534946891541186</v>
+        <v>1.534946114951027</v>
       </c>
       <c r="AX109" t="n">
         <v>0.3960970939331083</v>
       </c>
       <c r="AY109" t="n">
-        <v>855.4515404573906</v>
+        <v>855.4514250327325</v>
       </c>
       <c r="AZ109" t="inlineStr"/>
       <c r="BA109" t="n">
@@ -21641,10 +21645,10 @@
         </is>
       </c>
       <c r="Z110" t="n">
-        <v>1.160227417945862</v>
+        <v>1.160092830657959</v>
       </c>
       <c r="AA110" t="n">
-        <v>88291797356.10938</v>
+        <v>88281555438.5625</v>
       </c>
       <c r="AB110" t="inlineStr">
         <is>
@@ -21712,13 +21716,13 @@
         <v>0.8583092931365022</v>
       </c>
       <c r="AW110" t="n">
-        <v>0.7546123980858217</v>
+        <v>0.7546121975364353</v>
       </c>
       <c r="AX110" t="n">
         <v>0.5421563231244895</v>
       </c>
       <c r="AY110" t="n">
-        <v>0.1590857455921619</v>
+        <v>0.1590856580756304</v>
       </c>
       <c r="AZ110" t="inlineStr"/>
       <c r="BA110" t="n">
@@ -21871,13 +21875,13 @@
         <v>184.09619140625</v>
       </c>
       <c r="AL111" t="n">
-        <v>94.14984893798828</v>
+        <v>94.14984130859375</v>
       </c>
       <c r="AM111" t="n">
         <v>-0.1179610852215612</v>
       </c>
       <c r="AN111" t="n">
-        <v>0.724697455327453</v>
+        <v>0.7246975950876178</v>
       </c>
       <c r="AO111" t="n">
         <v>60.40415900751429</v>
@@ -21901,16 +21905,16 @@
         <v>0.4812569783626304</v>
       </c>
       <c r="AV111" t="n">
-        <v>0.707938894972072</v>
+        <v>0.70793875791478</v>
       </c>
       <c r="AW111" t="n">
-        <v>4.135520330887824</v>
+        <v>4.13551940152004</v>
       </c>
       <c r="AX111" t="n">
         <v>0.5272574571895901</v>
       </c>
       <c r="AY111" t="n">
-        <v>7.502514084485943</v>
+        <v>7.502513235320702</v>
       </c>
       <c r="AZ111" t="inlineStr"/>
       <c r="BA111" t="n">
@@ -22067,13 +22071,13 @@
         <v>785.1200561523438</v>
       </c>
       <c r="AL112" t="n">
-        <v>375.6900634765625</v>
+        <v>375.6901245117188</v>
       </c>
       <c r="AM112" t="n">
         <v>-0.1713623770125597</v>
       </c>
       <c r="AN112" t="n">
-        <v>0.7316934365245205</v>
+        <v>0.7316931551911221</v>
       </c>
       <c r="AO112" t="n">
         <v>53.45888465826619</v>
@@ -22097,10 +22101,10 @@
         <v>0.1641931124209326</v>
       </c>
       <c r="AV112" t="n">
-        <v>0.6711170303664067</v>
+        <v>0.6711168993688965</v>
       </c>
       <c r="AW112" t="n">
-        <v>4.652982663346365</v>
+        <v>4.652983412851675</v>
       </c>
       <c r="AX112" t="n">
         <v>0.4801838637494129</v>
@@ -22248,16 +22252,16 @@
         <v>277.0487933349609</v>
       </c>
       <c r="AG113" t="n">
-        <v>239.6324000549317</v>
+        <v>239.6324010467529</v>
       </c>
       <c r="AH113" t="n">
         <v>-0.03013469586866502</v>
       </c>
       <c r="AI113" t="n">
-        <v>0.1213008430639444</v>
+        <v>0.1213008384229608</v>
       </c>
       <c r="AJ113" t="n">
-        <v>0.1561407942809578</v>
+        <v>0.1561407894957743</v>
       </c>
       <c r="AK113" t="n">
         <v>330.5873718261719</v>
@@ -22293,16 +22297,16 @@
         <v>0.4228328260364922</v>
       </c>
       <c r="AV113" t="n">
-        <v>0.4952999524564978</v>
+        <v>0.495299825484198</v>
       </c>
       <c r="AW113" t="n">
-        <v>0.6304384136859051</v>
+        <v>0.6304387156054703</v>
       </c>
       <c r="AX113" t="n">
         <v>0.5390933280379866</v>
       </c>
       <c r="AY113" t="n">
-        <v>391.7937545275893</v>
+        <v>391.7936518530633</v>
       </c>
       <c r="AZ113" t="inlineStr"/>
       <c r="BA113" t="n">
@@ -22413,7 +22417,7 @@
         </is>
       </c>
       <c r="X114" t="n">
-        <v>47365718016</v>
+        <v>47725150208</v>
       </c>
       <c r="Y114" t="inlineStr">
         <is>
@@ -22424,7 +22428,7 @@
         <v>1</v>
       </c>
       <c r="AA114" t="n">
-        <v>47365718016</v>
+        <v>47725150208</v>
       </c>
       <c r="AB114" t="inlineStr">
         <is>
@@ -22444,28 +22448,28 @@
         <v>63.44828910827637</v>
       </c>
       <c r="AG114" t="n">
-        <v>61.17890142440796</v>
+        <v>61.17890167236328</v>
       </c>
       <c r="AH114" t="n">
         <v>-0.0943806382798521</v>
       </c>
       <c r="AI114" t="n">
-        <v>-0.06078733441348805</v>
+        <v>-0.06078733822007443</v>
       </c>
       <c r="AJ114" t="n">
-        <v>0.03709428628221523</v>
+        <v>0.03709428207891885</v>
       </c>
       <c r="AK114" t="n">
         <v>75.72768402099609</v>
       </c>
       <c r="AL114" t="n">
-        <v>49.78788757324219</v>
+        <v>49.78789138793945</v>
       </c>
       <c r="AM114" t="n">
         <v>-0.2412286229624899</v>
       </c>
       <c r="AN114" t="n">
-        <v>0.1540959435152605</v>
+        <v>0.1540958550896108</v>
       </c>
       <c r="AO114" t="n">
         <v>35.60830479855863</v>
@@ -22486,19 +22490,19 @@
         <v>-0.1751305609353182</v>
       </c>
       <c r="AU114" t="n">
-        <v>0.03992854130266998</v>
+        <v>0.03992861309887497</v>
       </c>
       <c r="AV114" t="n">
-        <v>-0.06350310460147512</v>
+        <v>-0.06350316282615642</v>
       </c>
       <c r="AW114" t="n">
         <v>0.07433489180473041</v>
       </c>
       <c r="AX114" t="n">
-        <v>0.08595428014442108</v>
+        <v>0.08595420185239799</v>
       </c>
       <c r="AY114" t="n">
-        <v>4.215002885290093</v>
+        <v>4.21500378805288</v>
       </c>
       <c r="AZ114" t="inlineStr"/>
       <c r="BA114" t="n">
@@ -22836,16 +22840,16 @@
         <v>61.02492607116699</v>
       </c>
       <c r="AG116" t="n">
-        <v>56.37644330978394</v>
+        <v>56.37644315719604</v>
       </c>
       <c r="AH116" t="n">
         <v>-0.1433009075942481</v>
       </c>
       <c r="AI116" t="n">
-        <v>-0.07266234423440721</v>
+        <v>-0.07266234172448471</v>
       </c>
       <c r="AJ116" t="n">
-        <v>0.08245434597283885</v>
+        <v>0.0824543489025984</v>
       </c>
       <c r="AK116" t="n">
         <v>86.98540496826172</v>
@@ -22884,13 +22888,13 @@
         <v>0.1660412987041053</v>
       </c>
       <c r="AW116" t="n">
-        <v>-0.4940093615494184</v>
+        <v>-0.4940092868237982</v>
       </c>
       <c r="AX116" t="n">
         <v>0.4172553934738501</v>
       </c>
       <c r="AY116" t="n">
-        <v>29.09113703929774</v>
+        <v>29.09113497462275</v>
       </c>
       <c r="AZ116" t="inlineStr"/>
       <c r="BA116" t="n">
@@ -23082,7 +23086,7 @@
         <v>0.03549680509580733</v>
       </c>
       <c r="AY117" t="n">
-        <v>18.37840791748473</v>
+        <v>18.37841674139106</v>
       </c>
       <c r="AZ117" t="inlineStr"/>
       <c r="BA117" t="n">
@@ -23224,16 +23228,16 @@
         <v>1318.587006835937</v>
       </c>
       <c r="AG118" t="n">
-        <v>1254.920339355469</v>
+        <v>1254.920336303711</v>
       </c>
       <c r="AH118" t="n">
         <v>-0.06380090616872336</v>
       </c>
       <c r="AI118" t="n">
-        <v>-0.01630412527099312</v>
+        <v>-0.01630412287880811</v>
       </c>
       <c r="AJ118" t="n">
-        <v>0.05073363263294328</v>
+        <v>0.05073363518815288</v>
       </c>
       <c r="AK118" t="n">
         <v>1687.3154296875</v>
@@ -23269,16 +23273,16 @@
         <v>0.1769211315774069</v>
       </c>
       <c r="AV118" t="n">
-        <v>0.4792092304377549</v>
+        <v>0.4792093386215719</v>
       </c>
       <c r="AW118" t="n">
-        <v>1.549541387677451</v>
+        <v>1.549541226984376</v>
       </c>
       <c r="AX118" t="n">
         <v>0.3230825046483616</v>
       </c>
       <c r="AY118" t="n">
-        <v>146.0532033949273</v>
+        <v>146.0531532769928</v>
       </c>
       <c r="AZ118" t="inlineStr"/>
       <c r="BA118" t="n">
@@ -23612,16 +23616,16 @@
         <v>464.2001568603516</v>
       </c>
       <c r="AG120" t="n">
-        <v>443.1174645996094</v>
+        <v>443.1174650573731</v>
       </c>
       <c r="AH120" t="n">
         <v>-0.0467043526941372</v>
       </c>
       <c r="AI120" t="n">
-        <v>-0.001348345830777364</v>
+        <v>-0.001348346862437122</v>
       </c>
       <c r="AJ120" t="n">
-        <v>0.04757811177628035</v>
+        <v>0.04757811069407691</v>
       </c>
       <c r="AK120" t="n">
         <v>502.2725524902344</v>
@@ -23660,13 +23664,13 @@
         <v>0.07415410473978401</v>
       </c>
       <c r="AW120" t="n">
-        <v>1.351476109007468</v>
+        <v>1.35147553701611</v>
       </c>
       <c r="AX120" t="n">
         <v>0.1197111861506492</v>
       </c>
       <c r="AY120" t="n">
-        <v>496.5462932123036</v>
+        <v>496.5466266498429</v>
       </c>
       <c r="AZ120" t="inlineStr"/>
       <c r="BA120" t="n">
@@ -24050,7 +24054,7 @@
         <v>0.3443647918038379</v>
       </c>
       <c r="AY122" t="n">
-        <v>213.4564700086271</v>
+        <v>213.4564410460151</v>
       </c>
       <c r="AZ122" t="inlineStr"/>
       <c r="BA122" t="n">
@@ -24190,28 +24194,28 @@
         <v>278.7325991821289</v>
       </c>
       <c r="AG123" t="n">
-        <v>259.3688683319092</v>
+        <v>259.3688678741455</v>
       </c>
       <c r="AH123" t="n">
         <v>-0.07775409724993776</v>
       </c>
       <c r="AI123" t="n">
-        <v>-0.008901880893279923</v>
+        <v>-0.008901879144077141</v>
       </c>
       <c r="AJ123" t="n">
-        <v>0.0746571127628175</v>
+        <v>0.07465711465949476</v>
       </c>
       <c r="AK123" t="n">
         <v>376.1517333984375</v>
       </c>
       <c r="AL123" t="n">
-        <v>134.6916351318359</v>
+        <v>134.6916198730469</v>
       </c>
       <c r="AM123" t="n">
         <v>-0.3166055749999594</v>
       </c>
       <c r="AN123" t="n">
-        <v>0.908507512786402</v>
+        <v>0.9085077289952024</v>
       </c>
       <c r="AO123" t="n">
         <v>48.03408585654849</v>
@@ -24232,19 +24236,19 @@
         <v>-0.1510764554471811</v>
       </c>
       <c r="AU123" t="n">
-        <v>-0.006587415460754698</v>
+        <v>-0.00658729830195004</v>
       </c>
       <c r="AV123" t="n">
         <v>0.8962725001561778</v>
       </c>
       <c r="AW123" t="n">
-        <v>8.162433724991168</v>
+        <v>8.162434347889697</v>
       </c>
       <c r="AX123" t="n">
-        <v>0.4644647444818799</v>
+        <v>0.4644648717862903</v>
       </c>
       <c r="AY123" t="n">
-        <v>24.86858131847862</v>
+        <v>24.86858380110207</v>
       </c>
       <c r="AZ123" t="inlineStr"/>
       <c r="BA123" t="n">
@@ -24359,10 +24363,10 @@
         </is>
       </c>
       <c r="Z124" t="n">
-        <v>0.1032577827572823</v>
+        <v>0.1031555235385895</v>
       </c>
       <c r="AA124" t="n">
-        <v>2776431794.555283</v>
+        <v>2773682212.504578</v>
       </c>
       <c r="AB124" t="inlineStr">
         <is>
@@ -24436,7 +24440,7 @@
         <v>-0.2349132495901315</v>
       </c>
       <c r="AY124" t="n">
-        <v>1.361050054211353</v>
+        <v>1.361050342945241</v>
       </c>
       <c r="AZ124" t="inlineStr"/>
       <c r="BA124" t="n">
@@ -24857,10 +24861,10 @@
         </is>
       </c>
       <c r="Z127" t="n">
-        <v>1.160227417945862</v>
+        <v>1.160092830657959</v>
       </c>
       <c r="AA127" t="n">
-        <v>239583373528.7168</v>
+        <v>239555581670.0078</v>
       </c>
       <c r="AB127" t="inlineStr">
         <is>
@@ -24934,7 +24938,7 @@
         <v>0.1210134822666133</v>
       </c>
       <c r="AY127" t="n">
-        <v>26.83960539389182</v>
+        <v>26.83959701521436</v>
       </c>
       <c r="AZ127" t="inlineStr"/>
       <c r="BA127" t="n">
@@ -25045,7 +25049,7 @@
         </is>
       </c>
       <c r="X128" t="n">
-        <v>79690465280</v>
+        <v>79812878336</v>
       </c>
       <c r="Y128" t="inlineStr">
         <is>
@@ -25056,7 +25060,7 @@
         <v>1</v>
       </c>
       <c r="AA128" t="n">
-        <v>79690465280</v>
+        <v>79812878336</v>
       </c>
       <c r="AB128" t="inlineStr">
         <is>
@@ -25245,10 +25249,10 @@
         </is>
       </c>
       <c r="Z129" t="n">
-        <v>1.160227417945862</v>
+        <v>1.160092830657959</v>
       </c>
       <c r="AA129" t="n">
-        <v>17378225906.32654</v>
+        <v>17376210018.52979</v>
       </c>
       <c r="AB129" t="inlineStr">
         <is>
@@ -25259,7 +25263,7 @@
         <v>35996</v>
       </c>
       <c r="AD129" t="n">
-        <v>28.1</v>
+        <v>28.2</v>
       </c>
       <c r="AE129" t="n">
         <v>189.25</v>
@@ -25316,7 +25320,7 @@
         <v>0.6333027791932562</v>
       </c>
       <c r="AW129" t="n">
-        <v>2.432210443544038</v>
+        <v>2.432210206094146</v>
       </c>
       <c r="AX129" t="n">
         <v>0.2772843734130734</v>
@@ -25660,16 +25664,16 @@
         <v>418.9347991943359</v>
       </c>
       <c r="AG131" t="n">
-        <v>374.9871116638184</v>
+        <v>374.9871136474609</v>
       </c>
       <c r="AH131" t="n">
         <v>0.03414658096570089</v>
       </c>
       <c r="AI131" t="n">
-        <v>0.1553463486040587</v>
+        <v>0.1553463424923975</v>
       </c>
       <c r="AJ131" t="n">
-        <v>0.1171978613758793</v>
+        <v>0.1171978554660196</v>
       </c>
       <c r="AK131" t="n">
         <v>477.5700073242188</v>
@@ -25714,7 +25718,7 @@
         <v>0.3625300792233379</v>
       </c>
       <c r="AY131" t="n">
-        <v>137.7298218081567</v>
+        <v>137.7298535822063</v>
       </c>
       <c r="AZ131" t="inlineStr"/>
       <c r="BA131" t="n">
@@ -25906,7 +25910,7 @@
         <v>0.5000319113671245</v>
       </c>
       <c r="AY132" t="n">
-        <v>12.37537405716182</v>
+        <v>12.37537818801857</v>
       </c>
       <c r="AZ132" t="inlineStr"/>
       <c r="BA132" t="n">
@@ -26098,7 +26102,7 @@
         <v>1.938560260497212</v>
       </c>
       <c r="AY133" t="n">
-        <v>2.744905618827064</v>
+        <v>2.744906504955742</v>
       </c>
       <c r="AZ133" t="inlineStr"/>
       <c r="BA133" t="n">
@@ -26288,13 +26292,13 @@
         <v>1.586293904262781</v>
       </c>
       <c r="AW134" t="n">
-        <v>2.918339764377794</v>
+        <v>2.918339473014786</v>
       </c>
       <c r="AX134" t="n">
         <v>0.4064773229425358</v>
       </c>
       <c r="AY134" t="n">
-        <v>17.99113522447463</v>
+        <v>17.99114206882559</v>
       </c>
       <c r="AZ134" t="inlineStr"/>
       <c r="BA134" t="n">
@@ -26436,28 +26440,28 @@
         <v>516.4606408691407</v>
       </c>
       <c r="AG135" t="n">
-        <v>411.0397342681885</v>
+        <v>411.039734954834</v>
       </c>
       <c r="AH135" t="n">
         <v>-0.1161185304147133</v>
       </c>
       <c r="AI135" t="n">
-        <v>0.110573874438455</v>
+        <v>0.1105738725832315</v>
       </c>
       <c r="AJ135" t="n">
-        <v>0.2564737610796743</v>
+        <v>0.2564737589807238</v>
       </c>
       <c r="AK135" t="n">
         <v>722.2277221679688</v>
       </c>
       <c r="AL135" t="n">
-        <v>166.8769989013672</v>
+        <v>166.8770141601562</v>
       </c>
       <c r="AM135" t="n">
         <v>-0.3679417499177511</v>
       </c>
       <c r="AN135" t="n">
-        <v>1.735487773867409</v>
+        <v>1.735487523741703</v>
       </c>
       <c r="AO135" t="n">
         <v>35.03965121002578</v>
@@ -26481,16 +26485,16 @@
         <v>0.3396954758803989</v>
       </c>
       <c r="AV135" t="n">
-        <v>1.697707124676037</v>
+        <v>1.697707367940375</v>
       </c>
       <c r="AW135" t="n">
-        <v>2.502677306737371</v>
+        <v>2.502676486538888</v>
       </c>
       <c r="AX135" t="n">
-        <v>0.7038600440025082</v>
+        <v>0.7038602380851491</v>
       </c>
       <c r="AY135" t="n">
-        <v>6622.183376384152</v>
+        <v>6622.1826604182</v>
       </c>
       <c r="AZ135" t="inlineStr"/>
       <c r="BA135" t="n">
@@ -26605,10 +26609,10 @@
         </is>
       </c>
       <c r="Z136" t="n">
-        <v>1.160227417945862</v>
+        <v>1.160092830657959</v>
       </c>
       <c r="AA136" t="n">
-        <v>47050237869.20947</v>
+        <v>47044780004.81836</v>
       </c>
       <c r="AB136" t="inlineStr">
         <is>
@@ -26676,13 +26680,13 @@
         <v>0.8281034068089408</v>
       </c>
       <c r="AW136" t="n">
-        <v>1.676350418993946</v>
+        <v>1.676350155692504</v>
       </c>
       <c r="AX136" t="n">
         <v>0.5049338540377588</v>
       </c>
       <c r="AY136" t="n">
-        <v>281.4536760350092</v>
+        <v>281.4536302121961</v>
       </c>
       <c r="AZ136" t="inlineStr"/>
       <c r="BA136" t="n">
@@ -26824,16 +26828,16 @@
         <v>1738.094543457031</v>
       </c>
       <c r="AG137" t="n">
-        <v>1491.523651428223</v>
+        <v>1491.523657836914</v>
       </c>
       <c r="AH137" t="n">
         <v>-0.02289547181349294</v>
       </c>
       <c r="AI137" t="n">
-        <v>0.138634340261317</v>
+        <v>0.1386343353688999</v>
       </c>
       <c r="AJ137" t="n">
-        <v>0.1653147717722763</v>
+        <v>0.1653147667652199</v>
       </c>
       <c r="AK137" t="n">
         <v>1986.870361328125</v>
@@ -26872,13 +26876,13 @@
         <v>1.125803490281717</v>
       </c>
       <c r="AW137" t="n">
-        <v>1.074369858190369</v>
+        <v>1.074369394253185</v>
       </c>
       <c r="AX137" t="n">
         <v>0.4663067634362432</v>
       </c>
       <c r="AY137" t="n">
-        <v>964.0757791566708</v>
+        <v>964.0759099087381</v>
       </c>
       <c r="AZ137" t="inlineStr"/>
       <c r="BA137" t="n">
@@ -27020,28 +27024,28 @@
         <v>198.311156616211</v>
       </c>
       <c r="AG138" t="n">
-        <v>172.5825635528564</v>
+        <v>172.5825632095337</v>
       </c>
       <c r="AH138" t="n">
         <v>-0.0891082354018099</v>
       </c>
       <c r="AI138" t="n">
-        <v>0.04668742699678496</v>
+        <v>0.04668742907898604</v>
       </c>
       <c r="AJ138" t="n">
-        <v>0.1490799101235663</v>
+        <v>0.1490799124094593</v>
       </c>
       <c r="AK138" t="n">
         <v>301.3693542480469</v>
       </c>
       <c r="AL138" t="n">
-        <v>95.41329193115234</v>
+        <v>95.41328430175781</v>
       </c>
       <c r="AM138" t="n">
         <v>-0.4006026265000727</v>
       </c>
       <c r="AN138" t="n">
-        <v>0.8932372600663794</v>
+        <v>0.8932374114525736</v>
       </c>
       <c r="AO138" t="n">
         <v>46.71374727949298</v>
@@ -27065,7 +27069,7 @@
         <v>0.2763984165807265</v>
       </c>
       <c r="AV138" t="n">
-        <v>0.8932372600663794</v>
+        <v>0.8932374114525736</v>
       </c>
       <c r="AW138" t="n">
         <v>4.549091924116841</v>
@@ -27074,7 +27078,7 @@
         <v>0.4226327764177782</v>
       </c>
       <c r="AY138" t="n">
-        <v>2979.627872424193</v>
+        <v>2979.628422070165</v>
       </c>
       <c r="AZ138" t="inlineStr"/>
       <c r="BA138" t="n">
@@ -27412,28 +27416,28 @@
         <v>365.6934375</v>
       </c>
       <c r="AG140" t="n">
-        <v>320.3741926574707</v>
+        <v>320.3741924285889</v>
       </c>
       <c r="AH140" t="n">
         <v>0.03835607173208611</v>
       </c>
       <c r="AI140" t="n">
-        <v>0.1852390421056238</v>
+        <v>0.1852390429523827</v>
       </c>
       <c r="AJ140" t="n">
-        <v>0.1414572268340681</v>
+        <v>0.1414572276495485</v>
       </c>
       <c r="AK140" t="n">
         <v>483.6542053222656</v>
       </c>
       <c r="AL140" t="n">
-        <v>112.0230102539062</v>
+        <v>112.0230178833008</v>
       </c>
       <c r="AM140" t="n">
         <v>-0.2148936222570621</v>
       </c>
       <c r="AN140" t="n">
-        <v>2.389660752376205</v>
+        <v>2.389660521521335</v>
       </c>
       <c r="AO140" t="n">
         <v>51.48695142225591</v>
@@ -27457,7 +27461,7 @@
         <v>0.3267553938009435</v>
       </c>
       <c r="AV140" t="n">
-        <v>2.292277102995972</v>
+        <v>2.292276667434656</v>
       </c>
       <c r="AW140" t="n">
         <v>2.17550712852658</v>
@@ -27466,7 +27470,7 @@
         <v>0.8316063272566419</v>
       </c>
       <c r="AY140" t="n">
-        <v>340.0657929127381</v>
+        <v>340.0658659514395</v>
       </c>
       <c r="AZ140" t="inlineStr"/>
       <c r="BA140" t="n">
@@ -27577,7 +27581,7 @@
         </is>
       </c>
       <c r="X141" t="n">
-        <v>25761505280</v>
+        <v>25763864576</v>
       </c>
       <c r="Y141" t="inlineStr">
         <is>
@@ -27588,7 +27592,7 @@
         <v>1</v>
       </c>
       <c r="AA141" t="n">
-        <v>25761505280</v>
+        <v>25763864576</v>
       </c>
       <c r="AB141" t="inlineStr">
         <is>
@@ -28038,13 +28042,13 @@
         <v>1.277695401812586</v>
       </c>
       <c r="AW143" t="n">
-        <v>0.7043972594970211</v>
+        <v>0.7043974236211203</v>
       </c>
       <c r="AX143" t="n">
         <v>0.09450472038799984</v>
       </c>
       <c r="AY143" t="n">
-        <v>265.4230140951702</v>
+        <v>265.4229827649019</v>
       </c>
       <c r="AZ143" t="inlineStr"/>
       <c r="BA143" t="n">
@@ -28428,7 +28432,7 @@
         <v>0.2811255516943993</v>
       </c>
       <c r="AY145" t="n">
-        <v>25.61084050445034</v>
+        <v>25.61083822246127</v>
       </c>
       <c r="AZ145" t="inlineStr"/>
       <c r="BA145" t="n">
@@ -28570,16 +28574,16 @@
         <v>448.7317785644531</v>
       </c>
       <c r="AG146" t="n">
-        <v>261.1508752822876</v>
+        <v>261.1508754348755</v>
       </c>
       <c r="AH146" t="n">
         <v>0.2642072728661486</v>
       </c>
       <c r="AI146" t="n">
-        <v>1.172269104647416</v>
+        <v>1.17226910337818</v>
       </c>
       <c r="AJ146" t="n">
-        <v>0.7182855622421425</v>
+        <v>0.7182855612381649</v>
       </c>
       <c r="AK146" t="n">
         <v>567.2899780273438</v>
@@ -28618,13 +28622,13 @@
         <v>3.582586931511815</v>
       </c>
       <c r="AW146" t="n">
-        <v>11.683863339917</v>
+        <v>11.68386009443489</v>
       </c>
       <c r="AX146" t="n">
-        <v>3.479492581674595</v>
+        <v>3.479492851537152</v>
       </c>
       <c r="AY146" t="n">
-        <v>50.74863757254941</v>
+        <v>50.74862856881375</v>
       </c>
       <c r="AZ146" t="inlineStr"/>
       <c r="BA146" t="n">
@@ -28814,7 +28818,7 @@
         <v>1.549610310271502</v>
       </c>
       <c r="AW147" t="n">
-        <v>3.619799361917025</v>
+        <v>3.619799689728903</v>
       </c>
       <c r="AX147" t="n">
         <v>1.593015808988345</v>
@@ -29010,13 +29014,13 @@
         <v>0.3621345839635881</v>
       </c>
       <c r="AW148" t="n">
-        <v>1.135952676902177</v>
+        <v>1.135952438510717</v>
       </c>
       <c r="AX148" t="n">
         <v>0.2007632302274407</v>
       </c>
       <c r="AY148" t="n">
-        <v>46.28117395542905</v>
+        <v>46.28113745199876</v>
       </c>
       <c r="AZ148" t="inlineStr"/>
       <c r="BA148" t="n">
@@ -29202,13 +29206,13 @@
         <v>0.7561868864342607</v>
       </c>
       <c r="AW149" t="n">
-        <v>6.500129480875004</v>
+        <v>6.500128902481166</v>
       </c>
       <c r="AX149" t="n">
         <v>0.2406611047327465</v>
       </c>
       <c r="AY149" t="n">
-        <v>37.65078489504264</v>
+        <v>37.65078105494056</v>
       </c>
       <c r="AZ149" t="inlineStr"/>
       <c r="BA149" t="n">
@@ -29515,10 +29519,10 @@
         </is>
       </c>
       <c r="Z151" t="n">
-        <v>1.352887034416199</v>
+        <v>1.353033423423767</v>
       </c>
       <c r="AA151" t="n">
-        <v>162181692014.5586</v>
+        <v>162199240868.4805</v>
       </c>
       <c r="AB151" t="inlineStr">
         <is>
@@ -29586,13 +29590,13 @@
         <v>0.2873624475878274</v>
       </c>
       <c r="AW151" t="n">
-        <v>12.328143118832</v>
+        <v>12.32814405055286</v>
       </c>
       <c r="AX151" t="n">
         <v>0.2153045512002121</v>
       </c>
       <c r="AY151" t="n">
-        <v>10.68251806707193</v>
+        <v>10.68251591953522</v>
       </c>
       <c r="AZ151" t="inlineStr"/>
       <c r="BA151" t="n">
@@ -29778,13 +29782,13 @@
         <v>1.50081439757112</v>
       </c>
       <c r="AW152" t="n">
-        <v>6.914598463214</v>
+        <v>6.914599290767164</v>
       </c>
       <c r="AX152" t="n">
         <v>0.5825466534444343</v>
       </c>
       <c r="AY152" t="n">
-        <v>81.15411477648358</v>
+        <v>81.1541092036418</v>
       </c>
       <c r="AZ152" t="inlineStr"/>
       <c r="BA152" t="n">
@@ -29895,7 +29899,7 @@
         </is>
       </c>
       <c r="X153" t="n">
-        <v>26344310784</v>
+        <v>25939607552</v>
       </c>
       <c r="Y153" t="inlineStr">
         <is>
@@ -29906,7 +29910,7 @@
         <v>1</v>
       </c>
       <c r="AA153" t="n">
-        <v>26344310784</v>
+        <v>25939607552</v>
       </c>
       <c r="AB153" t="inlineStr">
         <is>
@@ -30170,13 +30174,13 @@
         <v>0.2865761534076094</v>
       </c>
       <c r="AW154" t="n">
-        <v>1.721691532166064</v>
+        <v>1.721691304280843</v>
       </c>
       <c r="AX154" t="n">
         <v>0.100798968347741</v>
       </c>
       <c r="AY154" t="n">
-        <v>676.0470361218443</v>
+        <v>676.0470912071983</v>
       </c>
       <c r="AZ154" t="inlineStr"/>
       <c r="BA154" t="n">
@@ -30362,13 +30366,13 @@
         <v>0.565029914610981</v>
       </c>
       <c r="AW155" t="n">
-        <v>1.926646775056136</v>
+        <v>1.926647038555185</v>
       </c>
       <c r="AX155" t="n">
         <v>0.4368063630303214</v>
       </c>
       <c r="AY155" t="n">
-        <v>7.158155374320971</v>
+        <v>7.158153838701823</v>
       </c>
       <c r="AZ155" t="inlineStr"/>
       <c r="BA155" t="n">
@@ -30554,13 +30558,13 @@
         <v>0.3705709815400917</v>
       </c>
       <c r="AW156" t="n">
-        <v>4.178462086134936</v>
+        <v>4.178462694139246</v>
       </c>
       <c r="AX156" t="n">
         <v>0.2666649052450922</v>
       </c>
       <c r="AY156" t="n">
-        <v>16.68945482445296</v>
+        <v>16.68945127710476</v>
       </c>
       <c r="AZ156" t="inlineStr"/>
       <c r="BA156" t="n">
@@ -30747,16 +30751,16 @@
         <v>0.4446488211799347</v>
       </c>
       <c r="AV157" t="n">
-        <v>0.6908229350234771</v>
+        <v>0.6908227405033824</v>
       </c>
       <c r="AW157" t="n">
-        <v>1.170217098450263</v>
+        <v>1.170216617759489</v>
       </c>
       <c r="AX157" t="n">
         <v>0.4881553908068952</v>
       </c>
       <c r="AY157" t="n">
-        <v>2262.673411334917</v>
+        <v>2262.673751818292</v>
       </c>
       <c r="AZ157" t="inlineStr"/>
       <c r="BA157" t="n">
@@ -31094,28 +31098,28 @@
         <v>322.106947631836</v>
       </c>
       <c r="AG159" t="n">
-        <v>294.9937574768066</v>
+        <v>294.9937591552734</v>
       </c>
       <c r="AH159" t="n">
         <v>-0.01250193790968179</v>
       </c>
       <c r="AI159" t="n">
-        <v>0.07826005978202466</v>
+        <v>0.07826005364689936</v>
       </c>
       <c r="AJ159" t="n">
-        <v>0.09191106410840244</v>
+        <v>0.09191105789560505</v>
       </c>
       <c r="AK159" t="n">
         <v>385.5466918945312</v>
       </c>
       <c r="AL159" t="n">
-        <v>192.3445281982422</v>
+        <v>192.3445129394531</v>
       </c>
       <c r="AM159" t="n">
         <v>-0.1749897139325516</v>
       </c>
       <c r="AN159" t="n">
-        <v>0.6536991696713756</v>
+        <v>0.6536993008601808</v>
       </c>
       <c r="AO159" t="n">
         <v>53.2750509174165</v>
@@ -31139,16 +31143,16 @@
         <v>0.2695813267060276</v>
       </c>
       <c r="AV159" t="n">
-        <v>0.4861247100031811</v>
+        <v>0.4861246040548293</v>
       </c>
       <c r="AW159" t="n">
-        <v>4.206783256118798</v>
+        <v>4.206784231521757</v>
       </c>
       <c r="AX159" t="n">
         <v>0.324183924424728</v>
       </c>
       <c r="AY159" t="n">
-        <v>429.5292887569382</v>
+        <v>429.5292540233918</v>
       </c>
       <c r="AZ159" t="inlineStr"/>
       <c r="BA159" t="n">
@@ -32572,16 +32576,16 @@
         <v>383.0855993652344</v>
       </c>
       <c r="AG5" t="n">
-        <v>369.4377291870117</v>
+        <v>369.437728729248</v>
       </c>
       <c r="AH5" t="n">
         <v>-0.05506761195360621</v>
       </c>
       <c r="AI5" t="n">
-        <v>-0.02015965984044532</v>
+        <v>-0.02015965862634261</v>
       </c>
       <c r="AJ5" t="n">
-        <v>0.03694227497623559</v>
+        <v>0.03694227626109226</v>
       </c>
       <c r="AK5" t="n">
         <v>480.8090515136719</v>
@@ -32617,16 +32621,16 @@
         <v>0.1277732642630893</v>
       </c>
       <c r="AV5" t="n">
-        <v>0.01393743323475483</v>
+        <v>0.01393734656336121</v>
       </c>
       <c r="AW5" t="n">
-        <v>6.989550400843566</v>
+        <v>6.989549055484776</v>
       </c>
       <c r="AX5" t="n">
         <v>0.0451742685812544</v>
       </c>
       <c r="AY5" t="n">
-        <v>317.7678861779656</v>
+        <v>317.7679865664864</v>
       </c>
       <c r="AZ5" t="inlineStr"/>
       <c r="BA5" t="n">
@@ -32989,13 +32993,13 @@
         <v>433.3299865722656</v>
       </c>
       <c r="AL7" t="n">
-        <v>114.9438400268555</v>
+        <v>114.94384765625</v>
       </c>
       <c r="AM7" t="n">
         <v>-0.3117946819704582</v>
       </c>
       <c r="AN7" t="n">
-        <v>1.594484412135762</v>
+        <v>1.594484239926934</v>
       </c>
       <c r="AO7" t="n">
         <v>42.17106145701388</v>
@@ -33019,7 +33023,7 @@
         <v>0.4063622593446763</v>
       </c>
       <c r="AV7" t="n">
-        <v>1.594484412135762</v>
+        <v>1.594484239926934</v>
       </c>
       <c r="AW7" t="n">
         <v>4.144068438445124</v>
@@ -33028,7 +33032,7 @@
         <v>0.6145445719687945</v>
       </c>
       <c r="AY7" t="n">
-        <v>1580.800987088059</v>
+        <v>1580.801237132436</v>
       </c>
       <c r="AZ7" t="inlineStr"/>
       <c r="BA7" t="n">
@@ -33176,28 +33180,28 @@
         <v>216.8398794555664</v>
       </c>
       <c r="AG8" t="n">
-        <v>154.7597800064087</v>
+        <v>154.7597797775269</v>
       </c>
       <c r="AH8" t="n">
         <v>0.08882188413084724</v>
       </c>
       <c r="AI8" t="n">
-        <v>0.5255902153242824</v>
+        <v>0.5255902175805527</v>
       </c>
       <c r="AJ8" t="n">
-        <v>0.4011384575927086</v>
+        <v>0.4011384596649212</v>
       </c>
       <c r="AK8" t="n">
         <v>316.3519592285156</v>
       </c>
       <c r="AL8" t="n">
-        <v>66.44841766357422</v>
+        <v>66.44842529296875</v>
       </c>
       <c r="AM8" t="n">
         <v>-0.2536793302014302</v>
       </c>
       <c r="AN8" t="n">
-        <v>2.553132104648163</v>
+        <v>2.553131696688959</v>
       </c>
       <c r="AO8" t="n">
         <v>49.56449814743989</v>
@@ -33221,16 +33225,16 @@
         <v>1.689238258735586</v>
       </c>
       <c r="AV8" t="n">
-        <v>2.553132104648163</v>
+        <v>2.553131696688959</v>
       </c>
       <c r="AW8" t="n">
-        <v>2.910343169222694</v>
+        <v>2.910344157443346</v>
       </c>
       <c r="AX8" t="n">
         <v>1.645110953951491</v>
       </c>
       <c r="AY8" t="n">
-        <v>18.46524987496561</v>
+        <v>18.46525905777374</v>
       </c>
       <c r="AZ8" t="inlineStr"/>
       <c r="BA8" t="n">
@@ -33343,7 +33347,7 @@
         </is>
       </c>
       <c r="X9" t="n">
-        <v>61045092352</v>
+        <v>57012838400</v>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
@@ -33354,7 +33358,7 @@
         <v>1</v>
       </c>
       <c r="AA9" t="n">
-        <v>61045092352</v>
+        <v>57012838400</v>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
@@ -33507,7 +33511,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.871026180220513</v>
+        <v>0.871026096865585</v>
       </c>
     </row>
   </sheetData>
@@ -33651,10 +33655,10 @@
         <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>12190.78075282894</v>
+        <v>12190.77929100673</v>
       </c>
       <c r="D2" t="n">
-        <v>1523.847594103618</v>
+        <v>1523.847411375841</v>
       </c>
       <c r="E2" t="n">
         <v>413.47350528</v>
@@ -33666,7 +33670,7 @@
         <v>72.5</v>
       </c>
       <c r="H2" t="n">
-        <v>93.08561365693356</v>
+        <v>93.0856176242997</v>
       </c>
       <c r="I2" t="n">
         <v>4</v>
@@ -33675,40 +33679,40 @@
         <v>0.5</v>
       </c>
       <c r="K2" t="n">
-        <v>0.6709867421147913</v>
+        <v>0.6709867594664729</v>
       </c>
       <c r="L2" t="n">
-        <v>0.3965746754673237</v>
+        <v>0.3965747448740503</v>
       </c>
       <c r="M2" t="n">
-        <v>0.3597824340552492</v>
+        <v>0.359782518485823</v>
       </c>
       <c r="N2" t="n">
-        <v>0.9311327650985878</v>
+        <v>0.9311327656361142</v>
       </c>
       <c r="O2" t="n">
         <v>0.4071691950025514</v>
       </c>
       <c r="P2" t="n">
-        <v>0.6051403772433395</v>
+        <v>0.6051404007361075</v>
       </c>
       <c r="Q2" t="n">
-        <v>3.91688886322037</v>
+        <v>3.916888550084762</v>
       </c>
       <c r="R2" t="n">
         <v>1.349969281217933</v>
       </c>
       <c r="S2" t="n">
-        <v>4.718670041067009</v>
+        <v>4.718668527007228</v>
       </c>
       <c r="T2" t="n">
-        <v>1312.339527894158</v>
+        <v>1312.339746936125</v>
       </c>
       <c r="U2" t="n">
-        <v>352.1804761743786</v>
+        <v>352.1805725015148</v>
       </c>
       <c r="V2" t="n">
-        <v>3907.357163111829</v>
+        <v>3907.358290807244</v>
       </c>
       <c r="W2" t="inlineStr">
         <is>
@@ -33726,10 +33730,10 @@
         <v>15</v>
       </c>
       <c r="C3" t="n">
-        <v>4137.936979341727</v>
+        <v>4137.933880773337</v>
       </c>
       <c r="D3" t="n">
-        <v>275.8624652894485</v>
+        <v>275.8622587182224</v>
       </c>
       <c r="E3" t="n">
         <v>59.365711872</v>
@@ -33741,7 +33745,7 @@
         <v>60</v>
       </c>
       <c r="H3" t="n">
-        <v>78.79478914374249</v>
+        <v>78.79478326196158</v>
       </c>
       <c r="I3" t="n">
         <v>3</v>
@@ -33750,40 +33754,40 @@
         <v>0.2</v>
       </c>
       <c r="K3" t="n">
-        <v>0.4898229874662344</v>
+        <v>0.4898230004050771</v>
       </c>
       <c r="L3" t="n">
         <v>0.4226327764177782</v>
       </c>
       <c r="M3" t="n">
-        <v>0.4364430473798321</v>
+        <v>0.4364428821145317</v>
       </c>
       <c r="N3" t="n">
-        <v>1.2001211395717</v>
+        <v>1.200121136844314</v>
       </c>
       <c r="O3" t="n">
         <v>1.125803490281717</v>
       </c>
       <c r="P3" t="n">
-        <v>0.9782694451279339</v>
+        <v>0.9782693722562313</v>
       </c>
       <c r="Q3" t="n">
-        <v>3.165919080318758</v>
+        <v>3.165918960699043</v>
       </c>
       <c r="R3" t="n">
-        <v>2.538017659458036</v>
+        <v>2.538017249358794</v>
       </c>
       <c r="S3" t="n">
-        <v>2.926358901994654</v>
+        <v>2.926360402218545</v>
       </c>
       <c r="T3" t="n">
-        <v>779.4917053236533</v>
+        <v>779.4917054350602</v>
       </c>
       <c r="U3" t="n">
         <v>34.5682251961798</v>
       </c>
       <c r="V3" t="n">
-        <v>987.4028473682696</v>
+        <v>987.4032228482602</v>
       </c>
       <c r="W3" t="inlineStr">
         <is>
@@ -33801,10 +33805,10 @@
         <v>16</v>
       </c>
       <c r="C4" t="n">
-        <v>1524.292433415551</v>
+        <v>1523.905279037473</v>
       </c>
       <c r="D4" t="n">
-        <v>95.26827708847195</v>
+        <v>95.24407993984207</v>
       </c>
       <c r="E4" t="n">
         <v>43.19344640535009</v>
@@ -33816,7 +33820,7 @@
         <v>72.5</v>
       </c>
       <c r="H4" t="n">
-        <v>78.36094208126632</v>
+        <v>78.35937055852584</v>
       </c>
       <c r="I4" t="n">
         <v>8</v>
@@ -33825,40 +33829,40 @@
         <v>0.5</v>
       </c>
       <c r="K4" t="n">
-        <v>0.589544509868914</v>
+        <v>0.5895445267353239</v>
       </c>
       <c r="L4" t="n">
         <v>0.3097017758417258</v>
       </c>
       <c r="M4" t="n">
-        <v>1.16092354104413</v>
+        <v>1.161142620263629</v>
       </c>
       <c r="N4" t="n">
-        <v>0.7680581462464452</v>
+        <v>0.7680581274671674</v>
       </c>
       <c r="O4" t="n">
-        <v>0.4481774767691958</v>
+        <v>0.4481774237950199</v>
       </c>
       <c r="P4" t="n">
-        <v>1.318976850299747</v>
+        <v>1.319338456014733</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.982273910829386</v>
+        <v>6.982273858526188</v>
       </c>
       <c r="R4" t="n">
-        <v>4.192622671126867</v>
+        <v>4.192623462830502</v>
       </c>
       <c r="S4" t="n">
-        <v>6.713950257038555</v>
+        <v>6.713260274420884</v>
       </c>
       <c r="T4" t="n">
-        <v>239.2660758722272</v>
+        <v>239.2660945400126</v>
       </c>
       <c r="U4" t="n">
-        <v>41.21351976685477</v>
+        <v>41.21351784680373</v>
       </c>
       <c r="V4" t="n">
-        <v>738.2490050212693</v>
+        <v>738.4248892035364</v>
       </c>
       <c r="W4" t="inlineStr">
         <is>
@@ -33876,10 +33880,10 @@
         <v>12</v>
       </c>
       <c r="C5" t="n">
-        <v>13629.14429489245</v>
+        <v>13625.11204094045</v>
       </c>
       <c r="D5" t="n">
-        <v>1135.762024574371</v>
+        <v>1135.426003411704</v>
       </c>
       <c r="E5" t="n">
         <v>352.277921792</v>
@@ -33891,7 +33895,7 @@
         <v>60</v>
       </c>
       <c r="H5" t="n">
-        <v>72.49281397139784</v>
+        <v>72.49651112987671</v>
       </c>
       <c r="I5" t="n">
         <v>3</v>
@@ -33900,40 +33904,40 @@
         <v>0.25</v>
       </c>
       <c r="K5" t="n">
-        <v>0.4413457406718749</v>
+        <v>0.4413457457575875</v>
       </c>
       <c r="L5" t="n">
         <v>0.06540306328984713</v>
       </c>
       <c r="M5" t="n">
-        <v>0.05570401844894451</v>
+        <v>0.05527766061705892</v>
       </c>
       <c r="N5" t="n">
-        <v>0.296900278856094</v>
+        <v>0.2969002845854155</v>
       </c>
       <c r="O5" t="n">
-        <v>-0.06838303687460001</v>
+        <v>-0.06838307217853407</v>
       </c>
       <c r="P5" t="n">
-        <v>0.1128468061360255</v>
+        <v>0.1124310824188258</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.6848646102631869</v>
+        <v>0.6848644808439774</v>
       </c>
       <c r="R5" t="n">
-        <v>0.5957424107014953</v>
+        <v>0.5957420485376483</v>
       </c>
       <c r="S5" t="n">
-        <v>0.8402232093297275</v>
+        <v>0.8402230732291365</v>
       </c>
       <c r="T5" t="n">
-        <v>1232.51772180392</v>
+        <v>1232.517700190867</v>
       </c>
       <c r="U5" t="n">
-        <v>13.16359193078881</v>
+        <v>13.16358934893154</v>
       </c>
       <c r="V5" t="n">
-        <v>2960.333170186414</v>
+        <v>2961.206350867455</v>
       </c>
       <c r="W5" t="inlineStr">
         <is>
@@ -33951,10 +33955,10 @@
         <v>7</v>
       </c>
       <c r="C6" t="n">
-        <v>231.9362371389691</v>
+        <v>231.9053659286043</v>
       </c>
       <c r="D6" t="n">
-        <v>33.13374816270987</v>
+        <v>33.12933798980061</v>
       </c>
       <c r="E6" t="n">
         <v>13.69463807880896</v>
@@ -33966,7 +33970,7 @@
         <v>60</v>
       </c>
       <c r="H6" t="n">
-        <v>70.82669960738517</v>
+        <v>70.83266873895568</v>
       </c>
       <c r="I6" t="n">
         <v>2</v>
@@ -33975,13 +33979,13 @@
         <v>0.2857142857142857</v>
       </c>
       <c r="K6" t="n">
-        <v>2.165106193336312</v>
+        <v>2.165106208789628</v>
       </c>
       <c r="L6" t="n">
         <v>1.737572926819951</v>
       </c>
       <c r="M6" t="n">
-        <v>2.02787597961992</v>
+        <v>2.028103337331895</v>
       </c>
       <c r="N6" t="n">
         <v>4.202511672332323</v>
@@ -33990,25 +33994,25 @@
         <v>4.609529296781873</v>
       </c>
       <c r="P6" t="n">
-        <v>3.953099797902925</v>
+        <v>3.953460533818736</v>
       </c>
       <c r="Q6" t="n">
-        <v>4.071652642093385</v>
+        <v>4.071652797164063</v>
       </c>
       <c r="R6" t="n">
-        <v>4.293791511379664</v>
+        <v>4.2937918326055</v>
       </c>
       <c r="S6" t="n">
-        <v>4.878164929091728</v>
+        <v>4.878675905976077</v>
       </c>
       <c r="T6" t="n">
-        <v>36.08832703933998</v>
+        <v>36.08832702368397</v>
       </c>
       <c r="U6" t="n">
-        <v>27.26115241316053</v>
+        <v>27.26115988990115</v>
       </c>
       <c r="V6" t="n">
-        <v>52.69022037473084</v>
+        <v>52.69677040618198</v>
       </c>
       <c r="W6" t="inlineStr">
         <is>
@@ -34026,13 +34030,13 @@
         <v>23</v>
       </c>
       <c r="C7" t="n">
-        <v>1613.251089258423</v>
+        <v>1613.533775513869</v>
       </c>
       <c r="D7" t="n">
-        <v>73.32959496629195</v>
+        <v>73.34244434153952</v>
       </c>
       <c r="E7" t="n">
-        <v>45.25196089720019</v>
+        <v>45.42917496051172</v>
       </c>
       <c r="F7" t="n">
         <v>50</v>
@@ -34041,7 +34045,7 @@
         <v>45</v>
       </c>
       <c r="H7" t="n">
-        <v>61.83746837221284</v>
+        <v>61.83252607370451</v>
       </c>
       <c r="I7" t="n">
         <v>4</v>
@@ -34050,40 +34054,40 @@
         <v>0.1739130434782609</v>
       </c>
       <c r="K7" t="n">
-        <v>0.3383509634097989</v>
+        <v>0.3383509656376347</v>
       </c>
       <c r="L7" t="n">
         <v>0.3436109529136453</v>
       </c>
       <c r="M7" t="n">
-        <v>0.3854070263661142</v>
+        <v>0.3853462076566503</v>
       </c>
       <c r="N7" t="n">
-        <v>0.5905843036214745</v>
+        <v>0.5905842879365669</v>
       </c>
       <c r="O7" t="n">
-        <v>0.4872545914471264</v>
+        <v>0.487254582052885</v>
       </c>
       <c r="P7" t="n">
-        <v>0.5334192553471209</v>
+        <v>0.5333010865767651</v>
       </c>
       <c r="Q7" t="n">
-        <v>2.552016965807692</v>
+        <v>2.552016937606695</v>
       </c>
       <c r="R7" t="n">
-        <v>1.443211500274327</v>
+        <v>1.443210825983568</v>
       </c>
       <c r="S7" t="n">
-        <v>2.274902911679122</v>
+        <v>2.274467134668301</v>
       </c>
       <c r="T7" t="n">
-        <v>172.6897857206239</v>
+        <v>172.6898133732471</v>
       </c>
       <c r="U7" t="n">
-        <v>26.97985917888818</v>
+        <v>26.97985938786241</v>
       </c>
       <c r="V7" t="n">
-        <v>336.6213533057638</v>
+        <v>336.5308756919588</v>
       </c>
       <c r="W7" t="inlineStr">
         <is>
@@ -34101,10 +34105,10 @@
         <v>13</v>
       </c>
       <c r="C8" t="n">
-        <v>4602.22810839565</v>
+        <v>4599.957495518493</v>
       </c>
       <c r="D8" t="n">
-        <v>383.5190090329708</v>
+        <v>383.3297912932077</v>
       </c>
       <c r="E8" t="n">
         <v>188.0718788466943</v>
@@ -34116,7 +34120,7 @@
         <v>60</v>
       </c>
       <c r="H8" t="n">
-        <v>60.58455697682687</v>
+        <v>60.58521379295658</v>
       </c>
       <c r="I8" t="n">
         <v>2</v>
@@ -34125,40 +34129,40 @@
         <v>0.1538461538461539</v>
       </c>
       <c r="K8" t="n">
-        <v>1.703449127764178</v>
+        <v>1.703449136548285</v>
       </c>
       <c r="L8" t="n">
-        <v>1.387121523685535</v>
+        <v>1.38712142664241</v>
       </c>
       <c r="M8" t="n">
-        <v>1.747155495872239</v>
+        <v>1.747380974371368</v>
       </c>
       <c r="N8" t="n">
-        <v>6.48007570960763</v>
+        <v>6.480075704566159</v>
       </c>
       <c r="O8" t="n">
-        <v>4.573525264594901</v>
+        <v>4.573525449804195</v>
       </c>
       <c r="P8" t="n">
-        <v>5.550249939627902</v>
+        <v>5.551013325612136</v>
       </c>
       <c r="Q8" t="n">
-        <v>6.647876629633302</v>
+        <v>6.647876562519857</v>
       </c>
       <c r="R8" t="n">
-        <v>5.196201099431143</v>
+        <v>5.196202186893917</v>
       </c>
       <c r="S8" t="n">
-        <v>8.671752177781782</v>
+        <v>8.672322781009521</v>
       </c>
       <c r="T8" t="n">
-        <v>289.0544938547952</v>
+        <v>289.0545165951464</v>
       </c>
       <c r="U8" t="n">
-        <v>52.07563850050028</v>
+        <v>52.07564197610581</v>
       </c>
       <c r="V8" t="n">
-        <v>350.3037036328843</v>
+        <v>350.4618415633592</v>
       </c>
       <c r="W8" t="inlineStr">
         <is>
@@ -34176,13 +34180,13 @@
         <v>2</v>
       </c>
       <c r="C9" t="n">
-        <v>49.476672</v>
+        <v>49.483311616</v>
       </c>
       <c r="D9" t="n">
-        <v>24.738336</v>
+        <v>24.741655808</v>
       </c>
       <c r="E9" t="n">
-        <v>24.738336</v>
+        <v>24.741655808</v>
       </c>
       <c r="F9" t="n">
         <v>32.5</v>
@@ -34191,7 +34195,7 @@
         <v>32.5</v>
       </c>
       <c r="H9" t="n">
-        <v>56.07208907826298</v>
+        <v>56.07261612100428</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -34206,34 +34210,34 @@
         <v>0.2086888575022282</v>
       </c>
       <c r="M9" t="n">
-        <v>0.7922410938185285</v>
+        <v>0.792254141324386</v>
       </c>
       <c r="N9" t="n">
-        <v>0.1177027172319359</v>
+        <v>0.1177026438643051</v>
       </c>
       <c r="O9" t="n">
-        <v>0.1177027172319359</v>
+        <v>0.1177026438643051</v>
       </c>
       <c r="P9" t="n">
-        <v>0.865976311948242</v>
+        <v>0.8659929061624907</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.19678205393756</v>
+        <v>0.1967819478660771</v>
       </c>
       <c r="R9" t="n">
-        <v>0.19678205393756</v>
+        <v>0.1967819478660771</v>
       </c>
       <c r="S9" t="n">
-        <v>0.19678205393756</v>
+        <v>0.1967819478660771</v>
       </c>
       <c r="T9" t="n">
-        <v>11.18996633546931</v>
+        <v>11.18996377409344</v>
       </c>
       <c r="U9" t="n">
-        <v>11.18996633546931</v>
+        <v>11.18996377409344</v>
       </c>
       <c r="V9" t="n">
-        <v>20.90518278636718</v>
+        <v>20.90539524963291</v>
       </c>
       <c r="W9" t="inlineStr">
         <is>
@@ -34251,13 +34255,13 @@
         <v>21</v>
       </c>
       <c r="C10" t="n">
-        <v>3374.754110557964</v>
+        <v>3383.339527092048</v>
       </c>
       <c r="D10" t="n">
-        <v>168.7377055278982</v>
+        <v>161.1114060520023</v>
       </c>
       <c r="E10" t="n">
-        <v>60.583256064</v>
+        <v>59.801288704</v>
       </c>
       <c r="F10" t="n">
         <v>63.33333333333334</v>
@@ -34266,7 +34270,7 @@
         <v>60</v>
       </c>
       <c r="H10" t="n">
-        <v>54.82451140604501</v>
+        <v>54.83736706675327</v>
       </c>
       <c r="I10" t="n">
         <v>4</v>
@@ -34275,40 +34279,40 @@
         <v>0.1904761904761905</v>
       </c>
       <c r="K10" t="n">
-        <v>0.5759919721231389</v>
+        <v>0.5759919850081432</v>
       </c>
       <c r="L10" t="n">
         <v>0.4868980908830125</v>
       </c>
       <c r="M10" t="n">
-        <v>0.3523511453505843</v>
+        <v>0.3518195682224436</v>
       </c>
       <c r="N10" t="n">
-        <v>1.063146081442765</v>
+        <v>1.063146061246367</v>
       </c>
       <c r="O10" t="n">
         <v>0.6655675527290204</v>
       </c>
       <c r="P10" t="n">
-        <v>0.609590065819857</v>
+        <v>0.6096063392269743</v>
       </c>
       <c r="Q10" t="n">
-        <v>6.625520550500855</v>
+        <v>6.625520515081964</v>
       </c>
       <c r="R10" t="n">
-        <v>3.558486571925111</v>
+        <v>3.558487044212144</v>
       </c>
       <c r="S10" t="n">
-        <v>7.657745754732154</v>
+        <v>7.651945742866662</v>
       </c>
       <c r="T10" t="n">
-        <v>184.1877557032243</v>
+        <v>184.1877811514381</v>
       </c>
       <c r="U10" t="n">
-        <v>26.37210534198059</v>
+        <v>26.37210225047868</v>
       </c>
       <c r="V10" t="n">
-        <v>296.4551300416551</v>
+        <v>295.8104122665402</v>
       </c>
       <c r="W10" t="inlineStr">
         <is>
@@ -34326,13 +34330,13 @@
         <v>4</v>
       </c>
       <c r="C11" t="n">
-        <v>412.8046345710433</v>
+        <v>412.8972398805376</v>
       </c>
       <c r="D11" t="n">
-        <v>103.2011586427608</v>
+        <v>103.2243099701344</v>
       </c>
       <c r="E11" t="n">
-        <v>77.921517568</v>
+        <v>77.982724096</v>
       </c>
       <c r="F11" t="n">
         <v>38.75</v>
@@ -34341,7 +34345,7 @@
         <v>42.5</v>
       </c>
       <c r="H11" t="n">
-        <v>50.99757695971361</v>
+        <v>50.99457348965004</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -34356,7 +34360,7 @@
         <v>0.02663109810363867</v>
       </c>
       <c r="M11" t="n">
-        <v>0.03694125008453546</v>
+        <v>0.03690337925337711</v>
       </c>
       <c r="N11" t="n">
         <v>0.134685515564421</v>
@@ -34365,25 +34369,25 @@
         <v>0.04481157110862455</v>
       </c>
       <c r="P11" t="n">
-        <v>0.07991811713046142</v>
+        <v>0.07983020669320683</v>
       </c>
       <c r="Q11" t="n">
-        <v>1.136432677134309</v>
+        <v>1.136432617771836</v>
       </c>
       <c r="R11" t="n">
         <v>0.9665450843868131</v>
       </c>
       <c r="S11" t="n">
-        <v>0.9685573540113112</v>
+        <v>0.9684695948998382</v>
       </c>
       <c r="T11" t="n">
-        <v>77.21336555814975</v>
+        <v>77.21336346348038</v>
       </c>
       <c r="U11" t="n">
         <v>69.16442964005671</v>
       </c>
       <c r="V11" t="n">
-        <v>56.18055322329502</v>
+        <v>56.20830643552128</v>
       </c>
       <c r="W11" t="inlineStr">
         <is>
@@ -34401,10 +34405,10 @@
         <v>10</v>
       </c>
       <c r="C12" t="n">
-        <v>2714.416308224</v>
+        <v>2714.398722048</v>
       </c>
       <c r="D12" t="n">
-        <v>271.4416308224</v>
+        <v>271.4398722048001</v>
       </c>
       <c r="E12" t="n">
         <v>97.74932787200001</v>
@@ -34416,7 +34420,7 @@
         <v>85</v>
       </c>
       <c r="H12" t="n">
-        <v>50.69100698709964</v>
+        <v>50.6905538968224</v>
       </c>
       <c r="I12" t="n">
         <v>6</v>
@@ -34425,40 +34429,40 @@
         <v>0.6</v>
       </c>
       <c r="K12" t="n">
-        <v>0.2742595356832438</v>
+        <v>0.2742595265859271</v>
       </c>
       <c r="L12" t="n">
         <v>0.1775795212671972</v>
       </c>
       <c r="M12" t="n">
-        <v>0.20383550068074</v>
+        <v>0.2038305059168966</v>
       </c>
       <c r="N12" t="n">
-        <v>0.225699630520207</v>
+        <v>0.2256996277691782</v>
       </c>
       <c r="O12" t="n">
         <v>0.06560570933348919</v>
       </c>
       <c r="P12" t="n">
-        <v>0.1776750410311326</v>
+        <v>0.177676711367178</v>
       </c>
       <c r="Q12" t="n">
-        <v>1.256263967273778</v>
+        <v>1.256264049824698</v>
       </c>
       <c r="R12" t="n">
         <v>0.3317662417195366</v>
       </c>
       <c r="S12" t="n">
-        <v>5.037664567095729</v>
+        <v>5.037699358189217</v>
       </c>
       <c r="T12" t="n">
-        <v>55.6770967733568</v>
+        <v>55.67712301632721</v>
       </c>
       <c r="U12" t="n">
         <v>7.59271739874022</v>
       </c>
       <c r="V12" t="n">
-        <v>221.4969213297414</v>
+        <v>221.4986524376581</v>
       </c>
       <c r="W12" t="inlineStr">
         <is>
@@ -34476,10 +34480,10 @@
         <v>19</v>
       </c>
       <c r="C13" t="n">
-        <v>1191.413651844698</v>
+        <v>1191.277611885394</v>
       </c>
       <c r="D13" t="n">
-        <v>62.70598167603675</v>
+        <v>62.69882167817867</v>
       </c>
       <c r="E13" t="n">
         <v>44.465762304</v>
@@ -34491,7 +34495,7 @@
         <v>15</v>
       </c>
       <c r="H13" t="n">
-        <v>34.46762295007122</v>
+        <v>34.47105453487822</v>
       </c>
       <c r="I13" t="n">
         <v>2</v>
@@ -34500,40 +34504,40 @@
         <v>0.1052631578947368</v>
       </c>
       <c r="K13" t="n">
-        <v>-0.06540896904097501</v>
+        <v>-0.06540897484491454</v>
       </c>
       <c r="L13" t="n">
         <v>-0.01907464793006219</v>
       </c>
       <c r="M13" t="n">
-        <v>0.09351373372913574</v>
+        <v>0.09352354624405375</v>
       </c>
       <c r="N13" t="n">
-        <v>0.01532909985003196</v>
+        <v>0.01532910982466073</v>
       </c>
       <c r="O13" t="n">
-        <v>0.01229280570979929</v>
+        <v>0.01229274024237026</v>
       </c>
       <c r="P13" t="n">
-        <v>0.1944066269645373</v>
+        <v>0.1943976984366987</v>
       </c>
       <c r="Q13" t="n">
-        <v>2.017432855145617</v>
+        <v>2.0174331021769</v>
       </c>
       <c r="R13" t="n">
-        <v>1.494203214971247</v>
+        <v>1.494203401687402</v>
       </c>
       <c r="S13" t="n">
-        <v>1.949875247575221</v>
+        <v>1.950012039372698</v>
       </c>
       <c r="T13" t="n">
-        <v>72.54939216523481</v>
+        <v>72.54939997376441</v>
       </c>
       <c r="U13" t="n">
-        <v>12.08738809441496</v>
+        <v>12.08738919527145</v>
       </c>
       <c r="V13" t="n">
-        <v>101.534047028156</v>
+        <v>101.5377223440939</v>
       </c>
       <c r="W13" t="inlineStr">
         <is>
@@ -34551,10 +34555,10 @@
         <v>10</v>
       </c>
       <c r="C14" t="n">
-        <v>2391.690062282029</v>
+        <v>2390.742322898027</v>
       </c>
       <c r="D14" t="n">
-        <v>239.1690062282028</v>
+        <v>239.0742322898028</v>
       </c>
       <c r="E14" t="n">
         <v>52.75461632</v>
@@ -34566,7 +34570,7 @@
         <v>42.5</v>
       </c>
       <c r="H14" t="n">
-        <v>13.69527572470557</v>
+        <v>13.70866486202596</v>
       </c>
       <c r="I14" t="n">
         <v>3</v>
@@ -34575,40 +34579,40 @@
         <v>0.3</v>
       </c>
       <c r="K14" t="n">
-        <v>0.09215426797619192</v>
+        <v>0.09215425490925286</v>
       </c>
       <c r="L14" t="n">
         <v>0.06752794862490252</v>
       </c>
       <c r="M14" t="n">
-        <v>-0.01376948154002711</v>
+        <v>-0.01373580694084171</v>
       </c>
       <c r="N14" t="n">
-        <v>0.1105527726016025</v>
+        <v>0.1105527721504644</v>
       </c>
       <c r="O14" t="n">
         <v>0.1500282396580679</v>
       </c>
       <c r="P14" t="n">
-        <v>0.196978711072755</v>
+        <v>0.1969551111543572</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.4710584900344388</v>
+        <v>0.4710585301668816</v>
       </c>
       <c r="R14" t="n">
-        <v>0.3165675856652247</v>
+        <v>0.3165677251425468</v>
       </c>
       <c r="S14" t="n">
-        <v>0.676724970224086</v>
+        <v>0.6767906014861454</v>
       </c>
       <c r="T14" t="n">
-        <v>15.80304839580905</v>
+        <v>15.80304387097797</v>
       </c>
       <c r="U14" t="n">
-        <v>3.304729100978502</v>
+        <v>3.304728893469109</v>
       </c>
       <c r="V14" t="n">
-        <v>2.731639254959604</v>
+        <v>2.732826727705612</v>
       </c>
       <c r="W14" t="inlineStr">
         <is>

</xml_diff>